<commit_message>
Starting last update in LA DW documentation - adding new tables and updatting tables and variables
</commit_message>
<xml_diff>
--- a/dw_spec_table_1.xlsx
+++ b/dw_spec_table_1.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29530"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29628"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Enrique Caro Molina\Desktop\LIVERAIM_DATAWAREHOUSE\dw_documentation\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4E529E5A-7C70-4721-94C4-EDF801C1E3E2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BD0E00F0-71C5-4792-A6EF-0CEDDF02998C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="33300" yWindow="1035" windowWidth="23235" windowHeight="12090" activeTab="5" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" firstSheet="1" activeTab="6" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="population" sheetId="1" r:id="rId1"/>
@@ -19,6 +19,7 @@
     <sheet name="demographics" sheetId="4" r:id="rId4"/>
     <sheet name="medical_history" sheetId="5" r:id="rId5"/>
     <sheet name="fibroscan" sheetId="6" r:id="rId6"/>
+    <sheet name="variables_desc" sheetId="7" r:id="rId7"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -41,7 +42,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="781" uniqueCount="266">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1125" uniqueCount="361">
   <si>
     <t>Liveraim name</t>
   </si>
@@ -268,18 +269,6 @@
     <t>cohort_id</t>
   </si>
   <si>
-    <t>id</t>
-  </si>
-  <si>
-    <t>Codigo_Muestras</t>
-  </si>
-  <si>
-    <t>code</t>
-  </si>
-  <si>
-    <t>Codi_mostra</t>
-  </si>
-  <si>
     <t>waist</t>
   </si>
   <si>
@@ -839,13 +828,325 @@
   </si>
   <si>
     <t>Obtained from melting the variables `te`, `cap`.</t>
+  </si>
+  <si>
+    <t>liveraim_name</t>
+  </si>
+  <si>
+    <t>data_type</t>
+  </si>
+  <si>
+    <t>Units/levels</t>
+  </si>
+  <si>
+    <t>panels</t>
+  </si>
+  <si>
+    <t>Description</t>
+  </si>
+  <si>
+    <t>string</t>
+  </si>
+  <si>
+    <t>all panels</t>
+  </si>
+  <si>
+    <t>Intra-cohort identification code.</t>
+  </si>
+  <si>
+    <t>population</t>
+  </si>
+  <si>
+    <t>Identifier for each cohort.</t>
+  </si>
+  <si>
+    <t>datetime64[ns]</t>
+  </si>
+  <si>
+    <t>date</t>
+  </si>
+  <si>
+    <t>all cohort-related tables</t>
+  </si>
+  <si>
+    <t>Date of visit 0.</t>
+  </si>
+  <si>
+    <t>0: Finished
+1: Ongoing
+2: Withdrawn</t>
+  </si>
+  <si>
+    <t>Status of the patients in the cohort. Finished if recruitment is complete, ongoing if still recruiting, withdrawn otherwise.</t>
+  </si>
+  <si>
+    <t>Date of birth of the patients (calculated using variables age and inclusion_date).</t>
+  </si>
+  <si>
+    <t>Cohort from which the patient originates.</t>
+  </si>
+  <si>
+    <t>Date when recruitment finished or last version date for withdrawn patients.</t>
+  </si>
+  <si>
+    <t>float64</t>
+  </si>
+  <si>
+    <t>years</t>
+  </si>
+  <si>
+    <t>demographics, population</t>
+  </si>
+  <si>
+    <t>Age at inclusion.</t>
+  </si>
+  <si>
+    <t>0: Caucasian
+1: Latin-American
+2: African
+3: Asian
+4: Mix
+5: Other</t>
+  </si>
+  <si>
+    <t>demographics</t>
+  </si>
+  <si>
+    <t>Ethnicity or continent of origin.</t>
+  </si>
+  <si>
+    <t>0: Female
+1: Male</t>
+  </si>
+  <si>
+    <t>Gender of the patient.</t>
+  </si>
+  <si>
+    <t>0: No
+1: Yes</t>
+  </si>
+  <si>
+    <t>medical_history</t>
+  </si>
+  <si>
+    <t>High blood pressure status.</t>
+  </si>
+  <si>
+    <t>Abdominal obesity status.</t>
+  </si>
+  <si>
+    <t>High triglycerides status.</t>
+  </si>
+  <si>
+    <t>COPD comorbidity.</t>
+  </si>
+  <si>
+    <t>1: Current smoker
+2: Prior smoking
+3: Non-smoker</t>
+  </si>
+  <si>
+    <t>Smoking history of the patient.</t>
+  </si>
+  <si>
+    <t>kg</t>
+  </si>
+  <si>
+    <t>physical_exam</t>
+  </si>
+  <si>
+    <t>Weight of the patient.</t>
+  </si>
+  <si>
+    <t>cm</t>
+  </si>
+  <si>
+    <t>Height of the patient.</t>
+  </si>
+  <si>
+    <t>kg/m²</t>
+  </si>
+  <si>
+    <t>Body mass index.</t>
+  </si>
+  <si>
+    <t>Hip circumference.</t>
+  </si>
+  <si>
+    <t>probe</t>
+  </si>
+  <si>
+    <t>0: M
+1: XL</t>
+  </si>
+  <si>
+    <t>Probe type used in FibroScan.</t>
+  </si>
+  <si>
+    <t>kPa</t>
+  </si>
+  <si>
+    <t>Median liver stiffness (kPa).</t>
+  </si>
+  <si>
+    <t>dB/m</t>
+  </si>
+  <si>
+    <t>CAP median.</t>
+  </si>
+  <si>
+    <t>mg/dL</t>
+  </si>
+  <si>
+    <t>blood_test</t>
+  </si>
+  <si>
+    <t>Creatinine (mg/dL).</t>
+  </si>
+  <si>
+    <t>C-reactive protein (CRP, mg/dL).</t>
+  </si>
+  <si>
+    <t>Glucose (mg/dL).</t>
+  </si>
+  <si>
+    <t>U/L</t>
+  </si>
+  <si>
+    <t>Aspartate aminotransferase (AST).</t>
+  </si>
+  <si>
+    <t>Alanine aminotransferase (ALT).</t>
+  </si>
+  <si>
+    <t>Gamma-glutamyl transferase (GGT).</t>
+  </si>
+  <si>
+    <t>Bilirubin (mg/dL).</t>
+  </si>
+  <si>
+    <t>Conjugated bilirubin (mg/dL).</t>
+  </si>
+  <si>
+    <t>Alkaline phosphatase (U/L).</t>
+  </si>
+  <si>
+    <t>g/L</t>
+  </si>
+  <si>
+    <t>Total proteins (g/L).</t>
+  </si>
+  <si>
+    <t>Albumin (g/L).</t>
+  </si>
+  <si>
+    <t>%</t>
+  </si>
+  <si>
+    <t>Hematocrit.</t>
+  </si>
+  <si>
+    <t>10^9/L</t>
+  </si>
+  <si>
+    <t>Platelet count.</t>
+  </si>
+  <si>
+    <t>ng/mL</t>
+  </si>
+  <si>
+    <t>Ferritin (ng/mL).</t>
+  </si>
+  <si>
+    <t>Transferrin saturation (%).</t>
+  </si>
+  <si>
+    <t>INR (International Normalized Ratio).</t>
+  </si>
+  <si>
+    <t>Total cholesterol (mg/dL).</t>
+  </si>
+  <si>
+    <t>HDL-cholesterol (mg/dL).</t>
+  </si>
+  <si>
+    <t>LDL-cholesterol (mg/dL).</t>
+  </si>
+  <si>
+    <t>Triglycerides (mg/dL).</t>
+  </si>
+  <si>
+    <t>0: Negative
+1: Positive</t>
+  </si>
+  <si>
+    <t>HCV antibody status.</t>
+  </si>
+  <si>
+    <t>HBs antigen status.</t>
+  </si>
+  <si>
+    <t>Medication for alcoholism treatment.</t>
+  </si>
+  <si>
+    <t>Glycated hemoglobin (%).</t>
+  </si>
+  <si>
+    <t>White cell count.</t>
+  </si>
+  <si>
+    <t>imc</t>
+  </si>
+  <si>
+    <t>Metabolic syndrome</t>
+  </si>
+  <si>
+    <t>Fibrosis etiology</t>
+  </si>
+  <si>
+    <t>Fibrosis etiology including CAP criteria</t>
+  </si>
+  <si>
+    <t>UBE/week</t>
+  </si>
+  <si>
+    <t>mmHg</t>
+  </si>
+  <si>
+    <t>Diastolic blood pressure</t>
+  </si>
+  <si>
+    <t>Systolic blood pressure</t>
+  </si>
+  <si>
+    <t>Diabetes Mellitus type 2</t>
+  </si>
+  <si>
+    <t>waist circumference</t>
+  </si>
+  <si>
+    <t>waist hip ratio</t>
+  </si>
+  <si>
+    <t>UBE per week</t>
+  </si>
+  <si>
+    <t>Whether a patient belongs to a cohort classified as at-risk or general population.</t>
+  </si>
+  <si>
+    <t>Alcohol overuse</t>
+  </si>
+  <si>
+    <t>0: No
+1: Yes
+2: Previous</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="4" x14ac:knownFonts="1">
+  <fonts count="5" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -875,6 +1176,13 @@
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color theme="0"/>
+      <name val="Calibri"/>
+      <family val="2"/>
     </font>
   </fonts>
   <fills count="4">
@@ -1065,7 +1373,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="19">
+  <cellXfs count="21">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
@@ -1106,24 +1414,68 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="2" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="104">
+  <dxfs count="111">
+    <dxf>
+      <font>
+        <b/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color theme="0"/>
+        <name val="Calibri"/>
+        <scheme val="none"/>
+      </font>
+      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
     <dxf>
       <font>
         <b val="0"/>
@@ -1158,54 +1510,6 @@
         <vertical/>
         <horizontal/>
       </border>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <i val="0"/>
-        <strike val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="10"/>
-        <color theme="1"/>
-        <name val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </font>
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-      <border diagonalUp="0" diagonalDown="0" outline="0">
-        <left style="thin">
-          <color rgb="FF000000"/>
-        </left>
-        <right style="thin">
-          <color rgb="FF000000"/>
-        </right>
-        <top/>
-        <bottom/>
-      </border>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="0"/>
-        <i val="0"/>
-        <strike val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="10"/>
-        <color theme="1"/>
-        <name val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </font>
-      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
     <dxf>
       <font>
@@ -1457,13 +1761,6 @@
     </dxf>
     <dxf>
       <border outline="0">
-        <bottom style="thin">
-          <color rgb="FF000000"/>
-        </bottom>
-      </border>
-    </dxf>
-    <dxf>
-      <border outline="0">
         <left style="thin">
           <color rgb="FF000000"/>
         </left>
@@ -1496,6 +1793,13 @@
         <scheme val="minor"/>
       </font>
       <alignment horizontal="general" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <border outline="0">
+        <bottom style="thin">
+          <color rgb="FF000000"/>
+        </bottom>
+      </border>
     </dxf>
     <dxf>
       <font>
@@ -1754,38 +2058,10 @@
       </border>
     </dxf>
     <dxf>
-      <alignment textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
       <border outline="0">
         <top style="thin">
           <color rgb="FF000000"/>
         </top>
-      </border>
-    </dxf>
-    <dxf>
-      <border outline="0">
-        <bottom style="thin">
-          <color rgb="FF000000"/>
-        </bottom>
       </border>
     </dxf>
     <dxf>
@@ -1822,6 +2098,13 @@
         <scheme val="minor"/>
       </font>
       <alignment horizontal="general" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <border outline="0">
+        <bottom style="thin">
+          <color rgb="FF000000"/>
+        </bottom>
+      </border>
     </dxf>
     <dxf>
       <font>
@@ -1851,6 +2134,27 @@
         <top/>
         <bottom/>
       </border>
+    </dxf>
+    <dxf>
+      <alignment textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
     <dxf>
       <font>
@@ -2080,41 +2384,10 @@
       </border>
     </dxf>
     <dxf>
-      <alignment textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
       <border outline="0">
         <top style="thin">
           <color rgb="FF000000"/>
         </top>
-      </border>
-    </dxf>
-    <dxf>
-      <border outline="0">
-        <bottom style="thin">
-          <color rgb="FF000000"/>
-        </bottom>
       </border>
     </dxf>
     <dxf>
@@ -2151,6 +2424,13 @@
         <scheme val="minor"/>
       </font>
       <alignment horizontal="general" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <border outline="0">
+        <bottom style="thin">
+          <color rgb="FF000000"/>
+        </bottom>
+      </border>
     </dxf>
     <dxf>
       <font>
@@ -2180,6 +2460,30 @@
         <top/>
         <bottom/>
       </border>
+    </dxf>
+    <dxf>
+      <alignment textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
     <dxf>
       <font>
@@ -2450,25 +2754,73 @@
     </dxf>
     <dxf>
       <border outline="0">
+        <left style="thin">
+          <color rgb="FF000000"/>
+        </left>
+        <right style="thin">
+          <color rgb="FF000000"/>
+        </right>
+        <top style="thin">
+          <color rgb="FF000000"/>
+        </top>
         <bottom style="thin">
           <color rgb="FF000000"/>
         </bottom>
       </border>
     </dxf>
     <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="10"/>
+        <color theme="1"/>
+        <name val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
+      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
       <border outline="0">
+        <bottom style="thin">
+          <color rgb="FF000000"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="10"/>
+        <color theme="1"/>
+        <name val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <border diagonalUp="0" diagonalDown="0" outline="0">
         <left style="thin">
           <color rgb="FF000000"/>
         </left>
         <right style="thin">
           <color rgb="FF000000"/>
         </right>
-        <top style="thin">
-          <color rgb="FF000000"/>
-        </top>
-        <bottom style="thin">
-          <color rgb="FF000000"/>
-        </bottom>
+        <top/>
+        <bottom/>
       </border>
     </dxf>
     <dxf>
@@ -2602,169 +2954,186 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="3" xr:uid="{3D7F8D19-C6A7-467C-A805-50BF0B2FBB1D}" name="Table3" displayName="Table3" ref="A15:E25" totalsRowShown="0" headerRowDxfId="103" dataDxfId="102">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="3" xr:uid="{3D7F8D19-C6A7-467C-A805-50BF0B2FBB1D}" name="Table3" displayName="Table3" ref="A15:E25" totalsRowShown="0" headerRowDxfId="110" dataDxfId="109">
   <autoFilter ref="A15:E25" xr:uid="{3D7F8D19-C6A7-467C-A805-50BF0B2FBB1D}"/>
   <tableColumns count="5">
-    <tableColumn id="1" xr3:uid="{D7DE8C30-4A0E-444A-BC0D-95A6FE053499}" name="Liveraim name" dataDxfId="101"/>
-    <tableColumn id="2" xr3:uid="{8F1F5A2D-41A8-4A63-8522-E2F9A8B92B2B}" name="SQL data type" dataDxfId="100"/>
-    <tableColumn id="3" xr3:uid="{0ED914BF-320F-439B-9A1D-E187A4253227}" name="data type" dataDxfId="99"/>
-    <tableColumn id="4" xr3:uid="{D4765889-C391-4FFA-8B1A-42C0076F212B}" name="calculated" dataDxfId="98"/>
-    <tableColumn id="5" xr3:uid="{FC8664C1-6A10-43DC-9C22-5EB32D2E3503}" name="Rule/Notes" dataDxfId="97"/>
+    <tableColumn id="1" xr3:uid="{D7DE8C30-4A0E-444A-BC0D-95A6FE053499}" name="Liveraim name" dataDxfId="108"/>
+    <tableColumn id="2" xr3:uid="{8F1F5A2D-41A8-4A63-8522-E2F9A8B92B2B}" name="SQL data type" dataDxfId="107"/>
+    <tableColumn id="3" xr3:uid="{0ED914BF-320F-439B-9A1D-E187A4253227}" name="data type" dataDxfId="106"/>
+    <tableColumn id="4" xr3:uid="{D4765889-C391-4FFA-8B1A-42C0076F212B}" name="calculated" dataDxfId="105"/>
+    <tableColumn id="5" xr3:uid="{FC8664C1-6A10-43DC-9C22-5EB32D2E3503}" name="Rule/Notes" dataDxfId="104"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium15" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table10.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="11" xr:uid="{3E3C6290-E528-462C-B2F0-866FDCBB9256}" name="Table11" displayName="Table11" ref="A17:G31" totalsRowShown="0" headerRowDxfId="14" dataDxfId="13" headerRowBorderDxfId="30" tableBorderDxfId="31" totalsRowBorderDxfId="29">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="11" xr:uid="{3E3C6290-E528-462C-B2F0-866FDCBB9256}" name="Table11" displayName="Table11" ref="A17:G31" totalsRowShown="0" headerRowDxfId="31" dataDxfId="29" headerRowBorderDxfId="30" tableBorderDxfId="28" totalsRowBorderDxfId="27">
   <autoFilter ref="A17:G31" xr:uid="{3E3C6290-E528-462C-B2F0-866FDCBB9256}"/>
   <tableColumns count="7">
-    <tableColumn id="1" xr3:uid="{5AD31C4F-391C-4CC6-A61C-1FF8E4B90C32}" name="Liveraim" dataDxfId="21"/>
-    <tableColumn id="2" xr3:uid="{19AF6362-4FA4-4C9E-AD6A-15EE74E1795E}" name="Liverscreen" dataDxfId="20"/>
-    <tableColumn id="3" xr3:uid="{EB056613-E4C3-4166-B457-C14DB7D12675}" name="Glucofib" dataDxfId="19"/>
-    <tableColumn id="4" xr3:uid="{155145D9-A088-4B20-8786-83FF2425367F}" name="Alcofib" dataDxfId="18"/>
-    <tableColumn id="5" xr3:uid="{34049428-62BE-471E-976B-B0D9AC0B2920}" name="Decide" dataDxfId="17"/>
-    <tableColumn id="6" xr3:uid="{6EE09425-EBDA-4C7C-A7CC-DEE61C40D496}" name="Marina" dataDxfId="16"/>
-    <tableColumn id="7" xr3:uid="{AF4785E2-1FCA-4B92-88AC-DD9C398FCAA9}" name="Metronord" dataDxfId="15"/>
+    <tableColumn id="1" xr3:uid="{5AD31C4F-391C-4CC6-A61C-1FF8E4B90C32}" name="Liveraim" dataDxfId="26"/>
+    <tableColumn id="2" xr3:uid="{19AF6362-4FA4-4C9E-AD6A-15EE74E1795E}" name="Liverscreen" dataDxfId="25"/>
+    <tableColumn id="3" xr3:uid="{EB056613-E4C3-4166-B457-C14DB7D12675}" name="Glucofib" dataDxfId="24"/>
+    <tableColumn id="4" xr3:uid="{155145D9-A088-4B20-8786-83FF2425367F}" name="Alcofib" dataDxfId="23"/>
+    <tableColumn id="5" xr3:uid="{34049428-62BE-471E-976B-B0D9AC0B2920}" name="Decide" dataDxfId="22"/>
+    <tableColumn id="6" xr3:uid="{6EE09425-EBDA-4C7C-A7CC-DEE61C40D496}" name="Marina" dataDxfId="21"/>
+    <tableColumn id="7" xr3:uid="{AF4785E2-1FCA-4B92-88AC-DD9C398FCAA9}" name="Metronord" dataDxfId="20"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium15" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table11.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="12" xr:uid="{5AAE420D-DAB7-4EEC-9020-4E3118DABE07}" name="Table12" displayName="Table12" ref="A13:H15" totalsRowShown="0" headerRowDxfId="1" dataDxfId="2" headerRowBorderDxfId="11" tableBorderDxfId="12" totalsRowBorderDxfId="10">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="12" xr:uid="{5AAE420D-DAB7-4EEC-9020-4E3118DABE07}" name="Table12" displayName="Table12" ref="A13:H15" totalsRowShown="0" headerRowDxfId="19" dataDxfId="17" headerRowBorderDxfId="18" tableBorderDxfId="16" totalsRowBorderDxfId="15">
   <autoFilter ref="A13:H15" xr:uid="{5AAE420D-DAB7-4EEC-9020-4E3118DABE07}"/>
   <tableColumns count="8">
-    <tableColumn id="1" xr3:uid="{00664429-9FEF-4AF6-A3E6-BBDA993381DC}" name="Liveraim" dataDxfId="9"/>
-    <tableColumn id="2" xr3:uid="{F725255D-E953-4E1D-996B-31E7C24E3B5B}" name="Liverscreen" dataDxfId="8"/>
-    <tableColumn id="3" xr3:uid="{792E27B4-B9F3-48A9-8AE4-9FA268907D3B}" name="Glucofib" dataDxfId="7"/>
-    <tableColumn id="4" xr3:uid="{E3AC56AF-F2A1-41FB-B060-071EEF2135F5}" name="Alcofib" dataDxfId="6"/>
-    <tableColumn id="5" xr3:uid="{29F3B1B1-B765-41DC-AF41-A740F415CCCF}" name="Decide" dataDxfId="5"/>
-    <tableColumn id="6" xr3:uid="{7AC37435-5BE4-43D3-8672-BE18BBC47D9E}" name="Marina" dataDxfId="4"/>
-    <tableColumn id="7" xr3:uid="{BCDFA578-0248-4D11-AB75-D6604580CC0F}" name="Metronord" dataDxfId="3"/>
-    <tableColumn id="8" xr3:uid="{5E58108E-4739-42ED-8622-B36D89DDA63B}" name="Rule/Notes" dataDxfId="0"/>
+    <tableColumn id="1" xr3:uid="{00664429-9FEF-4AF6-A3E6-BBDA993381DC}" name="Liveraim" dataDxfId="14"/>
+    <tableColumn id="2" xr3:uid="{F725255D-E953-4E1D-996B-31E7C24E3B5B}" name="Liverscreen" dataDxfId="13"/>
+    <tableColumn id="3" xr3:uid="{792E27B4-B9F3-48A9-8AE4-9FA268907D3B}" name="Glucofib" dataDxfId="12"/>
+    <tableColumn id="4" xr3:uid="{E3AC56AF-F2A1-41FB-B060-071EEF2135F5}" name="Alcofib" dataDxfId="11"/>
+    <tableColumn id="5" xr3:uid="{29F3B1B1-B765-41DC-AF41-A740F415CCCF}" name="Decide" dataDxfId="10"/>
+    <tableColumn id="6" xr3:uid="{7AC37435-5BE4-43D3-8672-BE18BBC47D9E}" name="Marina" dataDxfId="9"/>
+    <tableColumn id="7" xr3:uid="{BCDFA578-0248-4D11-AB75-D6604580CC0F}" name="Metronord" dataDxfId="8"/>
+    <tableColumn id="8" xr3:uid="{5E58108E-4739-42ED-8622-B36D89DDA63B}" name="Rule/Notes" dataDxfId="7"/>
+  </tableColumns>
+  <tableStyleInfo name="TableStyleMedium15" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
+</table>
+</file>
+
+<file path=xl/tables/table12.xml><?xml version="1.0" encoding="utf-8"?>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="8" xr:uid="{94155B57-6209-4706-A84E-E6AA4B9B0C8A}" name="Table8" displayName="Table8" ref="A1:E60" totalsRowShown="0" headerRowDxfId="0" dataDxfId="1">
+  <autoFilter ref="A1:E60" xr:uid="{94155B57-6209-4706-A84E-E6AA4B9B0C8A}"/>
+  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:E60">
+    <sortCondition ref="D1:D60"/>
+  </sortState>
+  <tableColumns count="5">
+    <tableColumn id="1" xr3:uid="{3968AA77-89A5-4F78-8481-6C0A4679A711}" name="liveraim_name" dataDxfId="6"/>
+    <tableColumn id="2" xr3:uid="{8B304F56-D005-45A4-91EE-18BEF57D5CD1}" name="data_type" dataDxfId="5"/>
+    <tableColumn id="3" xr3:uid="{F135566C-F984-4758-B638-17736252C563}" name="Units/levels" dataDxfId="4"/>
+    <tableColumn id="4" xr3:uid="{808191B1-341A-4A1F-8B56-E78942D96BCF}" name="panels" dataDxfId="3"/>
+    <tableColumn id="5" xr3:uid="{C3095EA4-C4DF-4A56-A91B-020E12981701}" name="Description" dataDxfId="2"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium15" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="4" xr:uid="{EF5CF79F-A76D-4B1E-85FD-75991753497D}" name="Table4" displayName="Table4" ref="A1:G11" totalsRowShown="0" headerRowDxfId="96" dataDxfId="95">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="4" xr:uid="{EF5CF79F-A76D-4B1E-85FD-75991753497D}" name="Table4" displayName="Table4" ref="A1:G11" totalsRowShown="0" headerRowDxfId="103" dataDxfId="102">
   <autoFilter ref="A1:G11" xr:uid="{EF5CF79F-A76D-4B1E-85FD-75991753497D}"/>
   <tableColumns count="7">
-    <tableColumn id="1" xr3:uid="{6DCE9CA4-CEA1-4083-9FF6-AF108B62E1BC}" name="Liveraim name" dataDxfId="94"/>
-    <tableColumn id="2" xr3:uid="{223AD135-462B-4F84-B681-D752D50061B8}" name="Liverscreen name" dataDxfId="93"/>
-    <tableColumn id="3" xr3:uid="{51A8A5C6-609F-4B6C-9937-27DF2A53A648}" name="Alcofib name" dataDxfId="92"/>
-    <tableColumn id="4" xr3:uid="{E1FFC7F5-0D48-43FB-8E46-11BA2D29CB87}" name="Glucofib name" dataDxfId="91"/>
-    <tableColumn id="5" xr3:uid="{E6E90108-70B5-4852-9969-ABED859DB22F}" name="Decide name" dataDxfId="90"/>
-    <tableColumn id="6" xr3:uid="{1437B3EE-9FB0-4BEA-B8E2-86EF5C67025B}" name="Marina name" dataDxfId="89"/>
-    <tableColumn id="7" xr3:uid="{81C61AC6-CC68-440E-AB2F-E13A6FA9E989}" name="Galaald name" dataDxfId="88"/>
+    <tableColumn id="1" xr3:uid="{6DCE9CA4-CEA1-4083-9FF6-AF108B62E1BC}" name="Liveraim name" dataDxfId="101"/>
+    <tableColumn id="2" xr3:uid="{223AD135-462B-4F84-B681-D752D50061B8}" name="Liverscreen name" dataDxfId="100"/>
+    <tableColumn id="3" xr3:uid="{51A8A5C6-609F-4B6C-9937-27DF2A53A648}" name="Alcofib name" dataDxfId="99"/>
+    <tableColumn id="4" xr3:uid="{E1FFC7F5-0D48-43FB-8E46-11BA2D29CB87}" name="Glucofib name" dataDxfId="98"/>
+    <tableColumn id="5" xr3:uid="{E6E90108-70B5-4852-9969-ABED859DB22F}" name="Decide name" dataDxfId="97"/>
+    <tableColumn id="6" xr3:uid="{1437B3EE-9FB0-4BEA-B8E2-86EF5C67025B}" name="Marina name" dataDxfId="96"/>
+    <tableColumn id="7" xr3:uid="{81C61AC6-CC68-440E-AB2F-E13A6FA9E989}" name="Galaald name" dataDxfId="95"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium15" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="5" xr:uid="{DAED393B-A482-4058-B76E-7C28F20AF75D}" name="Table5" displayName="Table5" ref="A1:D12" totalsRowShown="0" headerRowDxfId="87" dataDxfId="86">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="5" xr:uid="{DAED393B-A482-4058-B76E-7C28F20AF75D}" name="Table5" displayName="Table5" ref="A1:D12" totalsRowShown="0" headerRowDxfId="94" dataDxfId="93">
   <autoFilter ref="A1:D12" xr:uid="{DAED393B-A482-4058-B76E-7C28F20AF75D}"/>
   <tableColumns count="4">
-    <tableColumn id="1" xr3:uid="{419BA3A1-A930-415B-9249-A70505329B55}" name="Liveraim name" dataDxfId="85"/>
-    <tableColumn id="2" xr3:uid="{39FFFF48-95FD-4A7B-8D94-62A65403C730}" name="Data type" dataDxfId="84"/>
-    <tableColumn id="3" xr3:uid="{3C597EBE-91C3-47D9-A06D-B1291F603660}" name="Secondary" dataDxfId="83"/>
-    <tableColumn id="4" xr3:uid="{3E9FCBED-023D-4146-9F34-92641715802E}" name="Rule/Notes" dataDxfId="82"/>
+    <tableColumn id="1" xr3:uid="{419BA3A1-A930-415B-9249-A70505329B55}" name="Liveraim name" dataDxfId="92"/>
+    <tableColumn id="2" xr3:uid="{39FFFF48-95FD-4A7B-8D94-62A65403C730}" name="Data type" dataDxfId="91"/>
+    <tableColumn id="3" xr3:uid="{3C597EBE-91C3-47D9-A06D-B1291F603660}" name="Secondary" dataDxfId="90"/>
+    <tableColumn id="4" xr3:uid="{3E9FCBED-023D-4146-9F34-92641715802E}" name="Rule/Notes" dataDxfId="89"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium15" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table4.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{A7178672-F88E-46B5-850E-9E6830651730}" name="Table1" displayName="Table1" ref="A15:I25" totalsRowShown="0" headerRowDxfId="81" dataDxfId="80">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{A7178672-F88E-46B5-850E-9E6830651730}" name="Table1" displayName="Table1" ref="A15:I25" totalsRowShown="0" headerRowDxfId="88" dataDxfId="87">
   <autoFilter ref="A15:I25" xr:uid="{A7178672-F88E-46B5-850E-9E6830651730}"/>
   <tableColumns count="9">
-    <tableColumn id="1" xr3:uid="{ACE7C3EE-5681-4438-89C3-AC808F3FC883}" name="Liveraim name" dataDxfId="79"/>
-    <tableColumn id="2" xr3:uid="{624CE68F-F0FC-47BA-8517-26350090AA0C}" name="Liverscreen name" dataDxfId="78"/>
-    <tableColumn id="3" xr3:uid="{1D7FD2D5-F284-47D3-B441-15AE4E5E12DB}" name="Alcofib name" dataDxfId="77"/>
-    <tableColumn id="4" xr3:uid="{30D5D9C4-5B5A-44AB-B4CD-BBDB7A659176}" name="Glucofib name" dataDxfId="76"/>
-    <tableColumn id="5" xr3:uid="{526EE2A7-6C11-4788-B360-E5AFA82930BE}" name="Decide name" dataDxfId="75"/>
-    <tableColumn id="6" xr3:uid="{85DF3E35-6C6F-407F-86A7-D21531A49D15}" name="Marina name" dataDxfId="74"/>
-    <tableColumn id="10" xr3:uid="{052F3FEE-EE8C-4801-A451-A699F0604F58}" name="Metronord" dataDxfId="73"/>
-    <tableColumn id="7" xr3:uid="{71378F90-1C75-4CD6-893D-858B42C21149}" name="Galaald name" dataDxfId="72"/>
-    <tableColumn id="9" xr3:uid="{B1253A0D-0CE0-4A90-81EC-BBE45C97CEA8}" name="Rule/Notes" dataDxfId="71"/>
+    <tableColumn id="1" xr3:uid="{ACE7C3EE-5681-4438-89C3-AC808F3FC883}" name="Liveraim name" dataDxfId="86"/>
+    <tableColumn id="2" xr3:uid="{624CE68F-F0FC-47BA-8517-26350090AA0C}" name="Liverscreen name" dataDxfId="85"/>
+    <tableColumn id="3" xr3:uid="{1D7FD2D5-F284-47D3-B441-15AE4E5E12DB}" name="Alcofib name" dataDxfId="84"/>
+    <tableColumn id="4" xr3:uid="{30D5D9C4-5B5A-44AB-B4CD-BBDB7A659176}" name="Glucofib name" dataDxfId="83"/>
+    <tableColumn id="5" xr3:uid="{526EE2A7-6C11-4788-B360-E5AFA82930BE}" name="Decide name" dataDxfId="82"/>
+    <tableColumn id="6" xr3:uid="{85DF3E35-6C6F-407F-86A7-D21531A49D15}" name="Marina name" dataDxfId="81"/>
+    <tableColumn id="10" xr3:uid="{052F3FEE-EE8C-4801-A451-A699F0604F58}" name="Metronord" dataDxfId="80"/>
+    <tableColumn id="7" xr3:uid="{71378F90-1C75-4CD6-893D-858B42C21149}" name="Galaald name" dataDxfId="79"/>
+    <tableColumn id="9" xr3:uid="{B1253A0D-0CE0-4A90-81EC-BBE45C97CEA8}" name="Rule/Notes" dataDxfId="78"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium15" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table5.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{C2246F92-3C6F-4EFB-A2EF-6C83982EF796}" name="Table53" displayName="Table53" ref="A1:D12" totalsRowShown="0" headerRowDxfId="66" dataDxfId="65">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{C2246F92-3C6F-4EFB-A2EF-6C83982EF796}" name="Table53" displayName="Table53" ref="A1:D12" totalsRowShown="0" headerRowDxfId="77" dataDxfId="76">
   <autoFilter ref="A1:D12" xr:uid="{C2246F92-3C6F-4EFB-A2EF-6C83982EF796}"/>
   <tableColumns count="4">
-    <tableColumn id="1" xr3:uid="{8488BC7C-2F31-4A72-A812-E06CC5E3B86E}" name="Liveraim name" dataDxfId="70"/>
-    <tableColumn id="2" xr3:uid="{D883FCE0-CFD8-4C88-A7B2-575396A879CA}" name="Data type" dataDxfId="69"/>
-    <tableColumn id="3" xr3:uid="{7CEFFAE3-E671-4F1B-8698-96550EE188CF}" name="Secondary" dataDxfId="68"/>
-    <tableColumn id="4" xr3:uid="{8BD4C8D5-3E18-4633-B4FD-3788EFD617D6}" name="Rule/Notes" dataDxfId="67"/>
+    <tableColumn id="1" xr3:uid="{8488BC7C-2F31-4A72-A812-E06CC5E3B86E}" name="Liveraim name" dataDxfId="75"/>
+    <tableColumn id="2" xr3:uid="{D883FCE0-CFD8-4C88-A7B2-575396A879CA}" name="Data type" dataDxfId="74"/>
+    <tableColumn id="3" xr3:uid="{7CEFFAE3-E671-4F1B-8698-96550EE188CF}" name="Secondary" dataDxfId="73"/>
+    <tableColumn id="4" xr3:uid="{8BD4C8D5-3E18-4633-B4FD-3788EFD617D6}" name="Rule/Notes" dataDxfId="72"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium15" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table6.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="6" xr:uid="{C0A23F03-DD3F-450F-81AC-2EDBB096B807}" name="Table6" displayName="Table6" ref="A16:H40" totalsRowShown="0" headerRowDxfId="53" dataDxfId="52" headerRowBorderDxfId="63" tableBorderDxfId="64" totalsRowBorderDxfId="62">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="6" xr:uid="{C0A23F03-DD3F-450F-81AC-2EDBB096B807}" name="Table6" displayName="Table6" ref="A16:H40" totalsRowShown="0" headerRowDxfId="71" dataDxfId="69" headerRowBorderDxfId="70" tableBorderDxfId="68" totalsRowBorderDxfId="67">
   <autoFilter ref="A16:H40" xr:uid="{C0A23F03-DD3F-450F-81AC-2EDBB096B807}"/>
   <tableColumns count="8">
-    <tableColumn id="1" xr3:uid="{0CF2EFCF-93B8-4C26-A2EA-7E46DC30E33F}" name="Liveraim" dataDxfId="61"/>
-    <tableColumn id="2" xr3:uid="{510636E5-4F01-45F9-A977-45CC2CE6E49C}" name="Liverscreen" dataDxfId="60"/>
-    <tableColumn id="3" xr3:uid="{0D023596-7339-4848-B398-AF8D5556F386}" name="Glucofib" dataDxfId="59"/>
-    <tableColumn id="4" xr3:uid="{4FEE6691-7864-45FC-B500-0D973A8DBF62}" name="Alcofib" dataDxfId="58"/>
-    <tableColumn id="5" xr3:uid="{FE603640-4DB3-4629-8CCD-9C5E51E8C484}" name="Decide" dataDxfId="57"/>
-    <tableColumn id="6" xr3:uid="{37A785CB-CD8B-467A-8499-A01860939C85}" name="Marina" dataDxfId="56"/>
-    <tableColumn id="7" xr3:uid="{1AF10A09-2F7C-4987-9228-11A8DCE043FF}" name="Metronord" dataDxfId="55"/>
-    <tableColumn id="8" xr3:uid="{33B0822D-68A7-4C5D-B051-388B9D425B7C}" name="Rules/Notes" dataDxfId="54"/>
+    <tableColumn id="1" xr3:uid="{0CF2EFCF-93B8-4C26-A2EA-7E46DC30E33F}" name="Liveraim" dataDxfId="66"/>
+    <tableColumn id="2" xr3:uid="{510636E5-4F01-45F9-A977-45CC2CE6E49C}" name="Liverscreen" dataDxfId="65"/>
+    <tableColumn id="3" xr3:uid="{0D023596-7339-4848-B398-AF8D5556F386}" name="Glucofib" dataDxfId="64"/>
+    <tableColumn id="4" xr3:uid="{4FEE6691-7864-45FC-B500-0D973A8DBF62}" name="Alcofib" dataDxfId="63"/>
+    <tableColumn id="5" xr3:uid="{FE603640-4DB3-4629-8CCD-9C5E51E8C484}" name="Decide" dataDxfId="62"/>
+    <tableColumn id="6" xr3:uid="{37A785CB-CD8B-467A-8499-A01860939C85}" name="Marina" dataDxfId="61"/>
+    <tableColumn id="7" xr3:uid="{1AF10A09-2F7C-4987-9228-11A8DCE043FF}" name="Metronord" dataDxfId="60"/>
+    <tableColumn id="8" xr3:uid="{33B0822D-68A7-4C5D-B051-388B9D425B7C}" name="Rules/Notes" dataDxfId="59"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium15" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table7.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="7" xr:uid="{F1658759-A43A-4D18-951E-CECA2AE32A6D}" name="Table7" displayName="Table7" ref="A1:F6" totalsRowShown="0" headerRowDxfId="42" dataDxfId="41">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="7" xr:uid="{F1658759-A43A-4D18-951E-CECA2AE32A6D}" name="Table7" displayName="Table7" ref="A1:F6" totalsRowShown="0" headerRowDxfId="58" dataDxfId="57">
   <autoFilter ref="A1:F6" xr:uid="{F1658759-A43A-4D18-951E-CECA2AE32A6D}"/>
   <tableColumns count="6">
-    <tableColumn id="1" xr3:uid="{157032E8-1023-4B47-A2FD-799BF93912C8}" name="Liveraim name" dataDxfId="48"/>
-    <tableColumn id="2" xr3:uid="{C97D4288-2E5C-4715-8C17-20F610111FB1}" name="SQL data type" dataDxfId="47"/>
-    <tableColumn id="3" xr3:uid="{1B6CFB06-13D1-45A2-A045-5E7CAEEEA840}" name="data type" dataDxfId="46"/>
-    <tableColumn id="4" xr3:uid="{464417B9-2150-414C-B0D9-010428D6FBA9}" name="Rule/Notes" dataDxfId="45"/>
-    <tableColumn id="5" xr3:uid="{B374587C-5969-47CB-B8C9-4103635C45BD}" name="Calculated" dataDxfId="44"/>
-    <tableColumn id="6" xr3:uid="{66412C9F-F468-4ED2-A12E-07AA300CEA7F}" name="Rules/Notes" dataDxfId="43"/>
+    <tableColumn id="1" xr3:uid="{157032E8-1023-4B47-A2FD-799BF93912C8}" name="Liveraim name" dataDxfId="56"/>
+    <tableColumn id="2" xr3:uid="{C97D4288-2E5C-4715-8C17-20F610111FB1}" name="SQL data type" dataDxfId="55"/>
+    <tableColumn id="3" xr3:uid="{1B6CFB06-13D1-45A2-A045-5E7CAEEEA840}" name="data type" dataDxfId="54"/>
+    <tableColumn id="4" xr3:uid="{464417B9-2150-414C-B0D9-010428D6FBA9}" name="Rule/Notes" dataDxfId="53"/>
+    <tableColumn id="5" xr3:uid="{B374587C-5969-47CB-B8C9-4103635C45BD}" name="Calculated" dataDxfId="52"/>
+    <tableColumn id="6" xr3:uid="{66412C9F-F468-4ED2-A12E-07AA300CEA7F}" name="Rules/Notes" dataDxfId="51"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium15" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table8.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="9" xr:uid="{273CBB74-0C71-46BF-A2F0-AC890186965A}" name="Table9" displayName="Table9" ref="A8:G13" totalsRowShown="0" headerRowDxfId="33" dataDxfId="32" headerRowBorderDxfId="50" tableBorderDxfId="51" totalsRowBorderDxfId="49">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="9" xr:uid="{273CBB74-0C71-46BF-A2F0-AC890186965A}" name="Table9" displayName="Table9" ref="A8:G13" totalsRowShown="0" headerRowDxfId="50" dataDxfId="48" headerRowBorderDxfId="49" tableBorderDxfId="47" totalsRowBorderDxfId="46">
   <autoFilter ref="A8:G13" xr:uid="{273CBB74-0C71-46BF-A2F0-AC890186965A}"/>
   <tableColumns count="7">
-    <tableColumn id="1" xr3:uid="{15CD80B5-F8F6-4106-B2E3-03089C70CD52}" name="Liveraim" dataDxfId="40"/>
-    <tableColumn id="2" xr3:uid="{EC0C2DD6-7E9C-4245-AD13-28CA9072B4C4}" name="Liverscreen" dataDxfId="39"/>
-    <tableColumn id="3" xr3:uid="{D9C4478E-942F-432C-BF2F-5678E98A6F24}" name="Glucofib" dataDxfId="38"/>
-    <tableColumn id="4" xr3:uid="{053AEF73-4666-4B31-BA7C-A8EAD38560CF}" name="Alcofib" dataDxfId="37"/>
-    <tableColumn id="5" xr3:uid="{9E364970-AD4E-4EE0-A05A-66B78E12F62E}" name="Decide" dataDxfId="36"/>
-    <tableColumn id="6" xr3:uid="{4EE35858-4E95-4EEC-BEFF-1200C3400BB5}" name="Marina" dataDxfId="35"/>
-    <tableColumn id="7" xr3:uid="{30619E3D-4A39-4BFE-A0AA-EE15910FE57E}" name="Metronord" dataDxfId="34"/>
+    <tableColumn id="1" xr3:uid="{15CD80B5-F8F6-4106-B2E3-03089C70CD52}" name="Liveraim" dataDxfId="45"/>
+    <tableColumn id="2" xr3:uid="{EC0C2DD6-7E9C-4245-AD13-28CA9072B4C4}" name="Liverscreen" dataDxfId="44"/>
+    <tableColumn id="3" xr3:uid="{D9C4478E-942F-432C-BF2F-5678E98A6F24}" name="Glucofib" dataDxfId="43"/>
+    <tableColumn id="4" xr3:uid="{053AEF73-4666-4B31-BA7C-A8EAD38560CF}" name="Alcofib" dataDxfId="42"/>
+    <tableColumn id="5" xr3:uid="{9E364970-AD4E-4EE0-A05A-66B78E12F62E}" name="Decide" dataDxfId="41"/>
+    <tableColumn id="6" xr3:uid="{4EE35858-4E95-4EEC-BEFF-1200C3400BB5}" name="Marina" dataDxfId="40"/>
+    <tableColumn id="7" xr3:uid="{30619E3D-4A39-4BFE-A0AA-EE15910FE57E}" name="Metronord" dataDxfId="39"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium15" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table9.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="10" xr:uid="{37B47D53-6619-403E-A6BE-D26135372257}" name="Table10" displayName="Table10" ref="A1:E15" totalsRowShown="0" headerRowDxfId="23" dataDxfId="22">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="10" xr:uid="{37B47D53-6619-403E-A6BE-D26135372257}" name="Table10" displayName="Table10" ref="A1:E15" totalsRowShown="0" headerRowDxfId="38" dataDxfId="37">
   <autoFilter ref="A1:E15" xr:uid="{37B47D53-6619-403E-A6BE-D26135372257}"/>
   <tableColumns count="5">
-    <tableColumn id="1" xr3:uid="{6DA11859-87C6-4742-B5C9-2A54C2CE7206}" name="Liveraim name" dataDxfId="28"/>
-    <tableColumn id="2" xr3:uid="{A441FFFA-7CD3-41F0-B3D5-B98D56A899F5}" name="SQL data type" dataDxfId="27"/>
-    <tableColumn id="3" xr3:uid="{8B221529-67BC-481D-8DCB-29141D988A0C}" name="Data type" dataDxfId="26"/>
-    <tableColumn id="4" xr3:uid="{01F5D246-D25D-4750-964B-7F5587EDAFA8}" name="secondary" dataDxfId="25"/>
-    <tableColumn id="5" xr3:uid="{435998E4-763C-4CAA-80CD-9FD3D3D106C6}" name="Rule/Notes" dataDxfId="24"/>
+    <tableColumn id="1" xr3:uid="{6DA11859-87C6-4742-B5C9-2A54C2CE7206}" name="Liveraim name" dataDxfId="36"/>
+    <tableColumn id="2" xr3:uid="{A441FFFA-7CD3-41F0-B3D5-B98D56A899F5}" name="SQL data type" dataDxfId="35"/>
+    <tableColumn id="3" xr3:uid="{8B221529-67BC-481D-8DCB-29141D988A0C}" name="Data type" dataDxfId="34"/>
+    <tableColumn id="4" xr3:uid="{01F5D246-D25D-4750-964B-7F5587EDAFA8}" name="secondary" dataDxfId="33"/>
+    <tableColumn id="5" xr3:uid="{435998E4-763C-4CAA-80CD-9FD3D3D106C6}" name="Rule/Notes" dataDxfId="32"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium15" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -3482,7 +3851,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{AA11D44F-3278-4E4D-8308-353744C21466}">
-  <dimension ref="A1:I25"/>
+  <dimension ref="A1:I35"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="3" width="21.21875" style="2" customWidth="1"/>
@@ -3665,7 +4034,7 @@
         <v>38</v>
       </c>
       <c r="G15" s="3" t="s">
-        <v>83</v>
+        <v>79</v>
       </c>
       <c r="H15" s="3" t="s">
         <v>39</v>
@@ -3694,7 +4063,7 @@
         <v>62</v>
       </c>
       <c r="G16" s="3" t="s">
-        <v>88</v>
+        <v>84</v>
       </c>
       <c r="H16" s="3" t="s">
         <v>60</v>
@@ -3723,7 +4092,7 @@
         <v>66</v>
       </c>
       <c r="G17" s="3" t="s">
-        <v>89</v>
+        <v>85</v>
       </c>
       <c r="H17" s="3" t="s">
         <v>64</v>
@@ -3781,7 +4150,7 @@
         <v>9</v>
       </c>
       <c r="G19" s="3" t="s">
-        <v>90</v>
+        <v>86</v>
       </c>
       <c r="H19" s="3" t="s">
         <v>71</v>
@@ -3792,25 +4161,25 @@
     </row>
     <row r="20" spans="1:9" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A20" s="3" t="s">
-        <v>79</v>
+        <v>75</v>
       </c>
       <c r="B20" s="3" t="s">
-        <v>79</v>
+        <v>75</v>
       </c>
       <c r="C20" s="3" t="s">
         <v>72</v>
       </c>
       <c r="D20" s="3" t="s">
-        <v>79</v>
+        <v>75</v>
       </c>
       <c r="E20" s="3" t="s">
-        <v>79</v>
+        <v>75</v>
       </c>
       <c r="F20" s="3" t="s">
         <v>73</v>
       </c>
       <c r="G20" s="3" t="s">
-        <v>91</v>
+        <v>87</v>
       </c>
       <c r="H20" s="3" t="s">
         <v>9</v>
@@ -3821,19 +4190,19 @@
     </row>
     <row r="21" spans="1:9" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A21" s="3" t="s">
-        <v>80</v>
+        <v>76</v>
       </c>
       <c r="B21" s="3" t="s">
-        <v>80</v>
+        <v>76</v>
       </c>
       <c r="C21" s="3" t="s">
         <v>9</v>
       </c>
       <c r="D21" s="3" t="s">
-        <v>80</v>
+        <v>76</v>
       </c>
       <c r="E21" s="3" t="s">
-        <v>80</v>
+        <v>76</v>
       </c>
       <c r="F21" s="3" t="s">
         <v>9</v>
@@ -3850,25 +4219,25 @@
     </row>
     <row r="22" spans="1:9" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A22" s="3" t="s">
+        <v>77</v>
+      </c>
+      <c r="B22" s="3" t="s">
+        <v>77</v>
+      </c>
+      <c r="C22" s="3" t="s">
+        <v>9</v>
+      </c>
+      <c r="D22" s="3" t="s">
+        <v>77</v>
+      </c>
+      <c r="E22" s="3" t="s">
+        <v>77</v>
+      </c>
+      <c r="F22" s="3" t="s">
+        <v>80</v>
+      </c>
+      <c r="G22" s="3" t="s">
         <v>81</v>
-      </c>
-      <c r="B22" s="3" t="s">
-        <v>81</v>
-      </c>
-      <c r="C22" s="3" t="s">
-        <v>9</v>
-      </c>
-      <c r="D22" s="3" t="s">
-        <v>81</v>
-      </c>
-      <c r="E22" s="3" t="s">
-        <v>81</v>
-      </c>
-      <c r="F22" s="3" t="s">
-        <v>84</v>
-      </c>
-      <c r="G22" s="3" t="s">
-        <v>85</v>
       </c>
       <c r="H22" s="3" t="s">
         <v>9</v>
@@ -3879,25 +4248,25 @@
     </row>
     <row r="23" spans="1:9" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A23" s="3" t="s">
+        <v>78</v>
+      </c>
+      <c r="B23" s="3" t="s">
+        <v>78</v>
+      </c>
+      <c r="C23" s="3" t="s">
+        <v>9</v>
+      </c>
+      <c r="D23" s="3" t="s">
+        <v>78</v>
+      </c>
+      <c r="E23" s="3" t="s">
+        <v>78</v>
+      </c>
+      <c r="F23" s="3" t="s">
         <v>82</v>
       </c>
-      <c r="B23" s="3" t="s">
-        <v>82</v>
-      </c>
-      <c r="C23" s="3" t="s">
-        <v>9</v>
-      </c>
-      <c r="D23" s="3" t="s">
-        <v>82</v>
-      </c>
-      <c r="E23" s="3" t="s">
-        <v>82</v>
-      </c>
-      <c r="F23" s="3" t="s">
-        <v>86</v>
-      </c>
       <c r="G23" s="3" t="s">
-        <v>87</v>
+        <v>83</v>
       </c>
       <c r="H23" s="3" t="s">
         <v>9</v>
@@ -3907,54 +4276,233 @@
       </c>
     </row>
     <row r="24" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A24" s="3" t="s">
-        <v>74</v>
-      </c>
-      <c r="B24" s="3" t="s">
+      <c r="A24" s="3"/>
+      <c r="B24" s="3"/>
+      <c r="C24" s="3"/>
+      <c r="D24" s="3"/>
+      <c r="E24" s="3"/>
+      <c r="F24" s="3"/>
+      <c r="G24" s="3"/>
+      <c r="H24" s="3"/>
+      <c r="I24" s="3"/>
+    </row>
+    <row r="25" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A25" s="3"/>
+      <c r="B25" s="3"/>
+      <c r="C25" s="3"/>
+      <c r="D25" s="3"/>
+      <c r="E25" s="3"/>
+      <c r="F25" s="3"/>
+      <c r="G25" s="3"/>
+      <c r="H25" s="3"/>
+      <c r="I25" s="3"/>
+    </row>
+    <row r="27" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A27" s="19" t="s">
+        <v>89</v>
+      </c>
+      <c r="B27" s="19" t="s">
+        <v>90</v>
+      </c>
+      <c r="C27" s="19" t="s">
+        <v>91</v>
+      </c>
+      <c r="D27" s="19" t="s">
+        <v>92</v>
+      </c>
+      <c r="E27" s="19" t="s">
+        <v>93</v>
+      </c>
+      <c r="F27" s="19" t="s">
+        <v>94</v>
+      </c>
+      <c r="G27" s="19" t="s">
+        <v>79</v>
+      </c>
+    </row>
+    <row r="28" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A28" s="4" t="s">
+        <v>60</v>
+      </c>
+      <c r="B28" s="4" t="s">
+        <v>60</v>
+      </c>
+      <c r="C28" s="4" t="s">
+        <v>60</v>
+      </c>
+      <c r="D28" s="4" t="s">
+        <v>61</v>
+      </c>
+      <c r="E28" s="4" t="s">
+        <v>60</v>
+      </c>
+      <c r="F28" s="4" t="s">
+        <v>62</v>
+      </c>
+      <c r="G28" s="4" t="s">
+        <v>84</v>
+      </c>
+    </row>
+    <row r="29" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A29" s="4" t="s">
+        <v>64</v>
+      </c>
+      <c r="B29" s="4" t="s">
+        <v>64</v>
+      </c>
+      <c r="C29" s="4" t="s">
+        <v>64</v>
+      </c>
+      <c r="D29" s="4" t="s">
+        <v>65</v>
+      </c>
+      <c r="E29" s="4" t="s">
+        <v>64</v>
+      </c>
+      <c r="F29" s="4" t="s">
+        <v>66</v>
+      </c>
+      <c r="G29" s="4" t="s">
+        <v>85</v>
+      </c>
+    </row>
+    <row r="30" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A30" s="4" t="s">
+        <v>67</v>
+      </c>
+      <c r="B30" s="4" t="s">
+        <v>67</v>
+      </c>
+      <c r="C30" s="4" t="s">
+        <v>67</v>
+      </c>
+      <c r="D30" s="4" t="s">
+        <v>68</v>
+      </c>
+      <c r="E30" s="4" t="s">
+        <v>67</v>
+      </c>
+      <c r="F30" s="4" t="s">
+        <v>69</v>
+      </c>
+      <c r="G30" s="4" t="s">
+        <v>346</v>
+      </c>
+    </row>
+    <row r="31" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A31" s="4" t="s">
+        <v>71</v>
+      </c>
+      <c r="B31" s="4" t="s">
+        <v>71</v>
+      </c>
+      <c r="C31" s="4" t="s">
+        <v>71</v>
+      </c>
+      <c r="D31" s="4" t="s">
+        <v>102</v>
+      </c>
+      <c r="E31" s="4" t="s">
+        <v>71</v>
+      </c>
+      <c r="F31" s="4" t="s">
+        <v>102</v>
+      </c>
+      <c r="G31" s="4" t="s">
+        <v>86</v>
+      </c>
+    </row>
+    <row r="32" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A32" s="4" t="s">
         <v>75</v>
       </c>
-      <c r="C24" s="3" t="s">
+      <c r="B32" s="4" t="s">
+        <v>75</v>
+      </c>
+      <c r="C32" s="4" t="s">
+        <v>75</v>
+      </c>
+      <c r="D32" s="4" t="s">
+        <v>72</v>
+      </c>
+      <c r="E32" s="4" t="s">
+        <v>75</v>
+      </c>
+      <c r="F32" s="4" t="s">
+        <v>73</v>
+      </c>
+      <c r="G32" s="4" t="s">
+        <v>87</v>
+      </c>
+    </row>
+    <row r="33" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A33" s="4" t="s">
         <v>76</v>
       </c>
-      <c r="D24" s="3" t="s">
+      <c r="B33" s="4" t="s">
+        <v>76</v>
+      </c>
+      <c r="C33" s="4" t="s">
+        <v>76</v>
+      </c>
+      <c r="D33" s="4" t="s">
+        <v>102</v>
+      </c>
+      <c r="E33" s="4" t="s">
+        <v>76</v>
+      </c>
+      <c r="F33" s="4" t="s">
+        <v>102</v>
+      </c>
+      <c r="G33" s="4" t="s">
+        <v>102</v>
+      </c>
+    </row>
+    <row r="34" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A34" s="4" t="s">
         <v>77</v>
       </c>
-      <c r="E24" s="3" t="s">
-        <v>75</v>
-      </c>
-      <c r="F24" s="3" t="s">
+      <c r="B34" s="4" t="s">
+        <v>77</v>
+      </c>
+      <c r="C34" s="4" t="s">
+        <v>77</v>
+      </c>
+      <c r="D34" s="4" t="s">
+        <v>102</v>
+      </c>
+      <c r="E34" s="4" t="s">
+        <v>77</v>
+      </c>
+      <c r="F34" s="4" t="s">
+        <v>80</v>
+      </c>
+      <c r="G34" s="4" t="s">
+        <v>81</v>
+      </c>
+    </row>
+    <row r="35" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A35" s="4" t="s">
         <v>78</v>
       </c>
-      <c r="G24" s="3"/>
-      <c r="H24" s="3" t="s">
-        <v>75</v>
-      </c>
-      <c r="I24" s="3"/>
-    </row>
-    <row r="25" spans="1:9" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="A25" s="3" t="s">
-        <v>29</v>
-      </c>
-      <c r="B25" s="3" t="s">
-        <v>20</v>
-      </c>
-      <c r="C25" s="3" t="s">
-        <v>21</v>
-      </c>
-      <c r="D25" s="3" t="s">
-        <v>20</v>
-      </c>
-      <c r="E25" s="3" t="s">
-        <v>42</v>
-      </c>
-      <c r="F25" s="3" t="s">
-        <v>43</v>
-      </c>
-      <c r="G25" s="3"/>
-      <c r="H25" s="3" t="s">
-        <v>44</v>
-      </c>
-      <c r="I25" s="3"/>
+      <c r="B35" s="4" t="s">
+        <v>78</v>
+      </c>
+      <c r="C35" s="4" t="s">
+        <v>78</v>
+      </c>
+      <c r="D35" s="4" t="s">
+        <v>102</v>
+      </c>
+      <c r="E35" s="4" t="s">
+        <v>78</v>
+      </c>
+      <c r="F35" s="4" t="s">
+        <v>82</v>
+      </c>
+      <c r="G35" s="4" t="s">
+        <v>83</v>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -3972,7 +4520,7 @@
   <cols>
     <col min="1" max="4" width="24.33203125" style="2" customWidth="1"/>
     <col min="5" max="7" width="14" customWidth="1"/>
-    <col min="8" max="8" width="32.109375" style="14" customWidth="1"/>
+    <col min="8" max="8" width="32.109375" customWidth="1"/>
     <col min="9" max="9" width="22.33203125" customWidth="1"/>
   </cols>
   <sheetData>
@@ -4026,7 +4574,7 @@
         <v>1</v>
       </c>
       <c r="D4" s="2" t="s">
-        <v>92</v>
+        <v>88</v>
       </c>
     </row>
     <row r="5" spans="1:8" ht="100.8" x14ac:dyDescent="0.3">
@@ -4040,7 +4588,7 @@
         <v>1</v>
       </c>
       <c r="D5" s="2" t="s">
-        <v>92</v>
+        <v>88</v>
       </c>
     </row>
     <row r="6" spans="1:8" ht="57.6" x14ac:dyDescent="0.3">
@@ -4117,51 +4665,51 @@
     </row>
     <row r="16" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A16" s="7" t="s">
+        <v>89</v>
+      </c>
+      <c r="B16" s="8" t="s">
+        <v>90</v>
+      </c>
+      <c r="C16" s="8" t="s">
+        <v>91</v>
+      </c>
+      <c r="D16" s="8" t="s">
+        <v>92</v>
+      </c>
+      <c r="E16" s="8" t="s">
         <v>93</v>
       </c>
-      <c r="B16" s="8" t="s">
+      <c r="F16" s="8" t="s">
         <v>94</v>
       </c>
-      <c r="C16" s="8" t="s">
-        <v>95</v>
-      </c>
-      <c r="D16" s="8" t="s">
-        <v>96</v>
-      </c>
-      <c r="E16" s="8" t="s">
-        <v>97</v>
-      </c>
-      <c r="F16" s="8" t="s">
-        <v>98</v>
-      </c>
       <c r="G16" s="9" t="s">
-        <v>83</v>
+        <v>79</v>
       </c>
       <c r="H16" s="8" t="s">
-        <v>202</v>
+        <v>198</v>
       </c>
     </row>
     <row r="17" spans="1:8" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A17" s="5" t="s">
+        <v>95</v>
+      </c>
+      <c r="B17" s="4" t="s">
+        <v>96</v>
+      </c>
+      <c r="C17" s="4" t="s">
+        <v>96</v>
+      </c>
+      <c r="D17" s="4" t="s">
+        <v>97</v>
+      </c>
+      <c r="E17" s="4" t="s">
+        <v>95</v>
+      </c>
+      <c r="F17" s="4" t="s">
+        <v>98</v>
+      </c>
+      <c r="G17" s="6" t="s">
         <v>99</v>
-      </c>
-      <c r="B17" s="4" t="s">
-        <v>100</v>
-      </c>
-      <c r="C17" s="4" t="s">
-        <v>100</v>
-      </c>
-      <c r="D17" s="4" t="s">
-        <v>101</v>
-      </c>
-      <c r="E17" s="4" t="s">
-        <v>99</v>
-      </c>
-      <c r="F17" s="4" t="s">
-        <v>102</v>
-      </c>
-      <c r="G17" s="6" t="s">
-        <v>103</v>
       </c>
       <c r="H17" s="3" t="s">
         <v>63</v>
@@ -4169,19 +4717,19 @@
     </row>
     <row r="18" spans="1:8" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A18" s="5" t="s">
-        <v>104</v>
+        <v>100</v>
       </c>
       <c r="B18" s="4" t="s">
-        <v>104</v>
+        <v>100</v>
       </c>
       <c r="C18" s="4" t="s">
-        <v>104</v>
+        <v>100</v>
       </c>
       <c r="D18" s="4" t="s">
-        <v>105</v>
+        <v>101</v>
       </c>
       <c r="E18" s="4" t="s">
-        <v>104</v>
+        <v>100</v>
       </c>
       <c r="F18" s="4" t="s">
         <v>9</v>
@@ -4195,25 +4743,25 @@
     </row>
     <row r="19" spans="1:8" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A19" s="5" t="s">
+        <v>103</v>
+      </c>
+      <c r="B19" s="4" t="s">
+        <v>104</v>
+      </c>
+      <c r="C19" s="4" t="s">
+        <v>104</v>
+      </c>
+      <c r="D19" s="4" t="s">
+        <v>105</v>
+      </c>
+      <c r="E19" s="4" t="s">
+        <v>103</v>
+      </c>
+      <c r="F19" s="4" t="s">
+        <v>106</v>
+      </c>
+      <c r="G19" s="6" t="s">
         <v>107</v>
-      </c>
-      <c r="B19" s="4" t="s">
-        <v>108</v>
-      </c>
-      <c r="C19" s="4" t="s">
-        <v>108</v>
-      </c>
-      <c r="D19" s="4" t="s">
-        <v>109</v>
-      </c>
-      <c r="E19" s="4" t="s">
-        <v>107</v>
-      </c>
-      <c r="F19" s="4" t="s">
-        <v>110</v>
-      </c>
-      <c r="G19" s="6" t="s">
-        <v>111</v>
       </c>
       <c r="H19" s="3" t="s">
         <v>63</v>
@@ -4221,25 +4769,25 @@
     </row>
     <row r="20" spans="1:8" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A20" s="5" t="s">
-        <v>112</v>
+        <v>108</v>
       </c>
       <c r="B20" s="4" t="s">
-        <v>112</v>
+        <v>108</v>
       </c>
       <c r="C20" s="4" t="s">
-        <v>112</v>
+        <v>108</v>
       </c>
       <c r="D20" s="4" t="s">
-        <v>113</v>
+        <v>109</v>
       </c>
       <c r="E20" s="4" t="s">
-        <v>112</v>
+        <v>108</v>
       </c>
       <c r="F20" s="4" t="s">
-        <v>114</v>
+        <v>110</v>
       </c>
       <c r="G20" s="6" t="s">
-        <v>115</v>
+        <v>111</v>
       </c>
       <c r="H20" s="3" t="s">
         <v>63</v>
@@ -4247,25 +4795,25 @@
     </row>
     <row r="21" spans="1:8" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A21" s="5" t="s">
-        <v>116</v>
+        <v>112</v>
       </c>
       <c r="B21" s="4" t="s">
-        <v>116</v>
+        <v>112</v>
       </c>
       <c r="C21" s="4" t="s">
-        <v>116</v>
+        <v>112</v>
       </c>
       <c r="D21" s="4" t="s">
-        <v>117</v>
+        <v>113</v>
       </c>
       <c r="E21" s="4" t="s">
-        <v>116</v>
+        <v>112</v>
       </c>
       <c r="F21" s="4" t="s">
-        <v>118</v>
+        <v>114</v>
       </c>
       <c r="G21" s="6" t="s">
-        <v>119</v>
+        <v>115</v>
       </c>
       <c r="H21" s="3" t="s">
         <v>63</v>
@@ -4273,25 +4821,25 @@
     </row>
     <row r="22" spans="1:8" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A22" s="5" t="s">
-        <v>120</v>
+        <v>116</v>
       </c>
       <c r="B22" s="4" t="s">
-        <v>120</v>
+        <v>116</v>
       </c>
       <c r="C22" s="4" t="s">
-        <v>120</v>
+        <v>116</v>
       </c>
       <c r="D22" s="4" t="s">
-        <v>121</v>
+        <v>117</v>
       </c>
       <c r="E22" s="4" t="s">
-        <v>120</v>
+        <v>116</v>
       </c>
       <c r="F22" s="4" t="s">
-        <v>122</v>
+        <v>118</v>
       </c>
       <c r="G22" s="6" t="s">
-        <v>120</v>
+        <v>116</v>
       </c>
       <c r="H22" s="3" t="s">
         <v>63</v>
@@ -4299,25 +4847,25 @@
     </row>
     <row r="23" spans="1:8" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A23" s="5" t="s">
+        <v>119</v>
+      </c>
+      <c r="B23" s="4" t="s">
+        <v>120</v>
+      </c>
+      <c r="C23" s="4" t="s">
+        <v>120</v>
+      </c>
+      <c r="D23" s="4" t="s">
+        <v>121</v>
+      </c>
+      <c r="E23" s="4" t="s">
+        <v>119</v>
+      </c>
+      <c r="F23" s="4" t="s">
+        <v>122</v>
+      </c>
+      <c r="G23" s="6" t="s">
         <v>123</v>
-      </c>
-      <c r="B23" s="4" t="s">
-        <v>124</v>
-      </c>
-      <c r="C23" s="4" t="s">
-        <v>124</v>
-      </c>
-      <c r="D23" s="4" t="s">
-        <v>125</v>
-      </c>
-      <c r="E23" s="4" t="s">
-        <v>123</v>
-      </c>
-      <c r="F23" s="4" t="s">
-        <v>126</v>
-      </c>
-      <c r="G23" s="6" t="s">
-        <v>127</v>
       </c>
       <c r="H23" s="3" t="s">
         <v>63</v>
@@ -4325,16 +4873,16 @@
     </row>
     <row r="24" spans="1:8" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A24" s="5" t="s">
-        <v>128</v>
+        <v>124</v>
       </c>
       <c r="B24" s="4" t="s">
-        <v>129</v>
+        <v>125</v>
       </c>
       <c r="C24" s="4" t="s">
-        <v>129</v>
+        <v>125</v>
       </c>
       <c r="D24" s="4" t="s">
-        <v>130</v>
+        <v>126</v>
       </c>
       <c r="E24" s="4" t="s">
         <v>9</v>
@@ -4351,25 +4899,25 @@
     </row>
     <row r="25" spans="1:8" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A25" s="5" t="s">
-        <v>131</v>
+        <v>127</v>
       </c>
       <c r="B25" s="4" t="s">
-        <v>131</v>
+        <v>127</v>
       </c>
       <c r="C25" s="4" t="s">
-        <v>131</v>
+        <v>127</v>
       </c>
       <c r="D25" s="4" t="s">
-        <v>132</v>
+        <v>128</v>
       </c>
       <c r="E25" s="4" t="s">
-        <v>131</v>
+        <v>127</v>
       </c>
       <c r="F25" s="4" t="s">
-        <v>133</v>
+        <v>129</v>
       </c>
       <c r="G25" s="6" t="s">
-        <v>134</v>
+        <v>130</v>
       </c>
       <c r="H25" s="3" t="s">
         <v>63</v>
@@ -4377,25 +4925,25 @@
     </row>
     <row r="26" spans="1:8" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A26" s="5" t="s">
+        <v>131</v>
+      </c>
+      <c r="B26" s="4" t="s">
+        <v>132</v>
+      </c>
+      <c r="C26" s="4" t="s">
+        <v>132</v>
+      </c>
+      <c r="D26" s="4" t="s">
+        <v>133</v>
+      </c>
+      <c r="E26" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="F26" s="4" t="s">
+        <v>134</v>
+      </c>
+      <c r="G26" s="6" t="s">
         <v>135</v>
-      </c>
-      <c r="B26" s="4" t="s">
-        <v>136</v>
-      </c>
-      <c r="C26" s="4" t="s">
-        <v>136</v>
-      </c>
-      <c r="D26" s="4" t="s">
-        <v>137</v>
-      </c>
-      <c r="E26" s="4" t="s">
-        <v>9</v>
-      </c>
-      <c r="F26" s="4" t="s">
-        <v>138</v>
-      </c>
-      <c r="G26" s="6" t="s">
-        <v>139</v>
       </c>
       <c r="H26" s="3" t="s">
         <v>63</v>
@@ -4403,25 +4951,25 @@
     </row>
     <row r="27" spans="1:8" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A27" s="5" t="s">
-        <v>140</v>
+        <v>136</v>
       </c>
       <c r="B27" s="4" t="s">
-        <v>140</v>
+        <v>136</v>
       </c>
       <c r="C27" s="4" t="s">
-        <v>140</v>
+        <v>136</v>
       </c>
       <c r="D27" s="4" t="s">
-        <v>141</v>
+        <v>137</v>
       </c>
       <c r="E27" s="4" t="s">
-        <v>140</v>
+        <v>136</v>
       </c>
       <c r="F27" s="4" t="s">
-        <v>142</v>
+        <v>138</v>
       </c>
       <c r="G27" s="6" t="s">
-        <v>140</v>
+        <v>136</v>
       </c>
       <c r="H27" s="3" t="s">
         <v>63</v>
@@ -4429,22 +4977,22 @@
     </row>
     <row r="28" spans="1:8" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A28" s="5" t="s">
-        <v>143</v>
+        <v>139</v>
       </c>
       <c r="B28" s="4" t="s">
-        <v>143</v>
+        <v>139</v>
       </c>
       <c r="C28" s="4" t="s">
-        <v>143</v>
+        <v>139</v>
       </c>
       <c r="D28" s="4" t="s">
-        <v>144</v>
+        <v>140</v>
       </c>
       <c r="E28" s="4" t="s">
-        <v>145</v>
+        <v>141</v>
       </c>
       <c r="F28" s="4" t="s">
-        <v>146</v>
+        <v>142</v>
       </c>
       <c r="G28" s="6" t="s">
         <v>9</v>
@@ -4455,25 +5003,25 @@
     </row>
     <row r="29" spans="1:8" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A29" s="5" t="s">
+        <v>143</v>
+      </c>
+      <c r="B29" s="4" t="s">
+        <v>143</v>
+      </c>
+      <c r="C29" s="4" t="s">
+        <v>143</v>
+      </c>
+      <c r="D29" s="4" t="s">
+        <v>144</v>
+      </c>
+      <c r="E29" s="4" t="s">
+        <v>145</v>
+      </c>
+      <c r="F29" s="4" t="s">
+        <v>146</v>
+      </c>
+      <c r="G29" s="6" t="s">
         <v>147</v>
-      </c>
-      <c r="B29" s="4" t="s">
-        <v>147</v>
-      </c>
-      <c r="C29" s="4" t="s">
-        <v>147</v>
-      </c>
-      <c r="D29" s="4" t="s">
-        <v>148</v>
-      </c>
-      <c r="E29" s="4" t="s">
-        <v>149</v>
-      </c>
-      <c r="F29" s="4" t="s">
-        <v>150</v>
-      </c>
-      <c r="G29" s="6" t="s">
-        <v>151</v>
       </c>
       <c r="H29" s="3" t="s">
         <v>63</v>
@@ -4481,25 +5029,25 @@
     </row>
     <row r="30" spans="1:8" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A30" s="5" t="s">
-        <v>152</v>
+        <v>148</v>
       </c>
       <c r="B30" s="4" t="s">
-        <v>152</v>
+        <v>148</v>
       </c>
       <c r="C30" s="4" t="s">
-        <v>152</v>
+        <v>148</v>
       </c>
       <c r="D30" s="4" t="s">
-        <v>153</v>
+        <v>149</v>
       </c>
       <c r="E30" s="4" t="s">
-        <v>154</v>
+        <v>150</v>
       </c>
       <c r="F30" s="4" t="s">
-        <v>155</v>
+        <v>151</v>
       </c>
       <c r="G30" s="6" t="s">
-        <v>154</v>
+        <v>150</v>
       </c>
       <c r="H30" s="3" t="s">
         <v>63</v>
@@ -4507,25 +5055,25 @@
     </row>
     <row r="31" spans="1:8" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A31" s="5" t="s">
-        <v>156</v>
+        <v>152</v>
       </c>
       <c r="B31" s="4" t="s">
-        <v>156</v>
+        <v>152</v>
       </c>
       <c r="C31" s="4" t="s">
-        <v>156</v>
+        <v>152</v>
       </c>
       <c r="D31" s="4" t="s">
-        <v>157</v>
+        <v>153</v>
       </c>
       <c r="E31" s="4" t="s">
-        <v>156</v>
+        <v>152</v>
       </c>
       <c r="F31" s="4" t="s">
-        <v>158</v>
+        <v>154</v>
       </c>
       <c r="G31" s="6" t="s">
-        <v>159</v>
+        <v>155</v>
       </c>
       <c r="H31" s="3" t="s">
         <v>63</v>
@@ -4533,25 +5081,25 @@
     </row>
     <row r="32" spans="1:8" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A32" s="5" t="s">
-        <v>160</v>
+        <v>156</v>
       </c>
       <c r="B32" s="4" t="s">
-        <v>160</v>
+        <v>156</v>
       </c>
       <c r="C32" s="4" t="s">
-        <v>160</v>
+        <v>156</v>
       </c>
       <c r="D32" s="4" t="s">
-        <v>161</v>
+        <v>157</v>
       </c>
       <c r="E32" s="4" t="s">
-        <v>160</v>
+        <v>156</v>
       </c>
       <c r="F32" s="4" t="s">
-        <v>162</v>
+        <v>158</v>
       </c>
       <c r="G32" s="6" t="s">
-        <v>163</v>
+        <v>159</v>
       </c>
       <c r="H32" s="3" t="s">
         <v>63</v>
@@ -4559,25 +5107,25 @@
     </row>
     <row r="33" spans="1:8" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A33" s="5" t="s">
+        <v>160</v>
+      </c>
+      <c r="B33" s="4" t="s">
+        <v>161</v>
+      </c>
+      <c r="C33" s="4" t="s">
+        <v>161</v>
+      </c>
+      <c r="D33" s="4" t="s">
+        <v>162</v>
+      </c>
+      <c r="E33" s="4" t="s">
+        <v>160</v>
+      </c>
+      <c r="F33" s="4" t="s">
+        <v>163</v>
+      </c>
+      <c r="G33" s="6" t="s">
         <v>164</v>
-      </c>
-      <c r="B33" s="4" t="s">
-        <v>165</v>
-      </c>
-      <c r="C33" s="4" t="s">
-        <v>165</v>
-      </c>
-      <c r="D33" s="4" t="s">
-        <v>166</v>
-      </c>
-      <c r="E33" s="4" t="s">
-        <v>164</v>
-      </c>
-      <c r="F33" s="4" t="s">
-        <v>167</v>
-      </c>
-      <c r="G33" s="6" t="s">
-        <v>168</v>
       </c>
       <c r="H33" s="3" t="s">
         <v>63</v>
@@ -4585,25 +5133,25 @@
     </row>
     <row r="34" spans="1:8" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A34" s="5" t="s">
-        <v>169</v>
+        <v>165</v>
       </c>
       <c r="B34" s="4" t="s">
-        <v>170</v>
+        <v>166</v>
       </c>
       <c r="C34" s="4" t="s">
-        <v>170</v>
+        <v>166</v>
       </c>
       <c r="D34" s="4" t="s">
-        <v>171</v>
+        <v>167</v>
       </c>
       <c r="E34" s="4" t="s">
-        <v>169</v>
+        <v>165</v>
       </c>
       <c r="F34" s="4" t="s">
-        <v>172</v>
+        <v>168</v>
       </c>
       <c r="G34" s="6" t="s">
-        <v>169</v>
+        <v>165</v>
       </c>
       <c r="H34" s="3" t="s">
         <v>63</v>
@@ -4611,25 +5159,25 @@
     </row>
     <row r="35" spans="1:8" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A35" s="5" t="s">
-        <v>173</v>
+        <v>169</v>
       </c>
       <c r="B35" s="4" t="s">
-        <v>174</v>
+        <v>170</v>
       </c>
       <c r="C35" s="4" t="s">
-        <v>174</v>
+        <v>170</v>
       </c>
       <c r="D35" s="4" t="s">
-        <v>175</v>
+        <v>171</v>
       </c>
       <c r="E35" s="4" t="s">
-        <v>173</v>
+        <v>169</v>
       </c>
       <c r="F35" s="4" t="s">
-        <v>176</v>
+        <v>172</v>
       </c>
       <c r="G35" s="6" t="s">
-        <v>173</v>
+        <v>169</v>
       </c>
       <c r="H35" s="3" t="s">
         <v>63</v>
@@ -4637,25 +5185,25 @@
     </row>
     <row r="36" spans="1:8" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A36" s="5" t="s">
+        <v>173</v>
+      </c>
+      <c r="B36" s="4" t="s">
+        <v>173</v>
+      </c>
+      <c r="C36" s="4" t="s">
+        <v>173</v>
+      </c>
+      <c r="D36" s="4" t="s">
+        <v>174</v>
+      </c>
+      <c r="E36" s="4" t="s">
+        <v>175</v>
+      </c>
+      <c r="F36" s="4" t="s">
+        <v>176</v>
+      </c>
+      <c r="G36" s="6" t="s">
         <v>177</v>
-      </c>
-      <c r="B36" s="4" t="s">
-        <v>177</v>
-      </c>
-      <c r="C36" s="4" t="s">
-        <v>177</v>
-      </c>
-      <c r="D36" s="4" t="s">
-        <v>178</v>
-      </c>
-      <c r="E36" s="4" t="s">
-        <v>179</v>
-      </c>
-      <c r="F36" s="4" t="s">
-        <v>180</v>
-      </c>
-      <c r="G36" s="6" t="s">
-        <v>181</v>
       </c>
       <c r="H36" s="3" t="s">
         <v>63</v>
@@ -4663,25 +5211,25 @@
     </row>
     <row r="37" spans="1:8" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A37" s="5" t="s">
+        <v>178</v>
+      </c>
+      <c r="B37" s="4" t="s">
+        <v>178</v>
+      </c>
+      <c r="C37" s="4" t="s">
+        <v>178</v>
+      </c>
+      <c r="D37" s="4" t="s">
+        <v>179</v>
+      </c>
+      <c r="E37" s="4" t="s">
+        <v>180</v>
+      </c>
+      <c r="F37" s="4" t="s">
+        <v>181</v>
+      </c>
+      <c r="G37" s="6" t="s">
         <v>182</v>
-      </c>
-      <c r="B37" s="4" t="s">
-        <v>182</v>
-      </c>
-      <c r="C37" s="4" t="s">
-        <v>182</v>
-      </c>
-      <c r="D37" s="4" t="s">
-        <v>183</v>
-      </c>
-      <c r="E37" s="4" t="s">
-        <v>184</v>
-      </c>
-      <c r="F37" s="4" t="s">
-        <v>185</v>
-      </c>
-      <c r="G37" s="6" t="s">
-        <v>186</v>
       </c>
       <c r="H37" s="3" t="s">
         <v>63</v>
@@ -4689,25 +5237,25 @@
     </row>
     <row r="38" spans="1:8" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A38" s="5" t="s">
+        <v>183</v>
+      </c>
+      <c r="B38" s="4" t="s">
+        <v>183</v>
+      </c>
+      <c r="C38" s="4" t="s">
+        <v>183</v>
+      </c>
+      <c r="D38" s="4" t="s">
+        <v>184</v>
+      </c>
+      <c r="E38" s="4" t="s">
+        <v>185</v>
+      </c>
+      <c r="F38" s="4" t="s">
+        <v>186</v>
+      </c>
+      <c r="G38" s="6" t="s">
         <v>187</v>
-      </c>
-      <c r="B38" s="4" t="s">
-        <v>187</v>
-      </c>
-      <c r="C38" s="4" t="s">
-        <v>187</v>
-      </c>
-      <c r="D38" s="4" t="s">
-        <v>188</v>
-      </c>
-      <c r="E38" s="4" t="s">
-        <v>189</v>
-      </c>
-      <c r="F38" s="4" t="s">
-        <v>190</v>
-      </c>
-      <c r="G38" s="6" t="s">
-        <v>191</v>
       </c>
       <c r="H38" s="3" t="s">
         <v>63</v>
@@ -4715,54 +5263,54 @@
     </row>
     <row r="39" spans="1:8" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A39" s="5" t="s">
+        <v>188</v>
+      </c>
+      <c r="B39" s="4" t="s">
+        <v>188</v>
+      </c>
+      <c r="C39" s="4" t="s">
+        <v>188</v>
+      </c>
+      <c r="D39" s="4" t="s">
+        <v>189</v>
+      </c>
+      <c r="E39" s="4" t="s">
+        <v>190</v>
+      </c>
+      <c r="F39" s="4" t="s">
+        <v>191</v>
+      </c>
+      <c r="G39" s="6" t="s">
         <v>192</v>
       </c>
-      <c r="B39" s="4" t="s">
-        <v>192</v>
-      </c>
-      <c r="C39" s="4" t="s">
-        <v>192</v>
-      </c>
-      <c r="D39" s="4" t="s">
-        <v>193</v>
-      </c>
-      <c r="E39" s="4" t="s">
-        <v>194</v>
-      </c>
-      <c r="F39" s="4" t="s">
-        <v>195</v>
-      </c>
-      <c r="G39" s="6" t="s">
-        <v>196</v>
-      </c>
       <c r="H39" s="3" t="s">
-        <v>203</v>
+        <v>199</v>
       </c>
     </row>
     <row r="40" spans="1:8" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A40" s="10" t="s">
+        <v>193</v>
+      </c>
+      <c r="B40" s="11" t="s">
+        <v>193</v>
+      </c>
+      <c r="C40" s="11" t="s">
+        <v>193</v>
+      </c>
+      <c r="D40" s="11" t="s">
+        <v>194</v>
+      </c>
+      <c r="E40" s="11" t="s">
+        <v>195</v>
+      </c>
+      <c r="F40" s="11" t="s">
+        <v>196</v>
+      </c>
+      <c r="G40" s="12" t="s">
         <v>197</v>
       </c>
-      <c r="B40" s="11" t="s">
-        <v>197</v>
-      </c>
-      <c r="C40" s="11" t="s">
-        <v>197</v>
-      </c>
-      <c r="D40" s="11" t="s">
-        <v>198</v>
-      </c>
-      <c r="E40" s="11" t="s">
+      <c r="H40" s="3" t="s">
         <v>199</v>
-      </c>
-      <c r="F40" s="11" t="s">
-        <v>200</v>
-      </c>
-      <c r="G40" s="12" t="s">
-        <v>201</v>
-      </c>
-      <c r="H40" s="3" t="s">
-        <v>203</v>
       </c>
     </row>
   </sheetData>
@@ -4798,10 +5346,10 @@
         <v>7</v>
       </c>
       <c r="E1" s="2" t="s">
-        <v>204</v>
+        <v>200</v>
       </c>
       <c r="F1" s="2" t="s">
-        <v>202</v>
+        <v>198</v>
       </c>
     </row>
     <row r="2" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
@@ -4849,7 +5397,7 @@
         <v>35</v>
       </c>
       <c r="C4" s="2" t="s">
-        <v>208</v>
+        <v>204</v>
       </c>
       <c r="D4" s="2" t="s">
         <v>9</v>
@@ -4872,18 +5420,18 @@
         <v>16</v>
       </c>
       <c r="D5" s="2" t="s">
-        <v>206</v>
+        <v>202</v>
       </c>
       <c r="E5" s="2" t="b">
         <v>0</v>
       </c>
       <c r="F5" s="2" t="s">
-        <v>212</v>
+        <v>208</v>
       </c>
     </row>
     <row r="6" spans="1:7" ht="57.6" x14ac:dyDescent="0.3">
       <c r="A6" s="2" t="s">
-        <v>205</v>
+        <v>201</v>
       </c>
       <c r="B6" s="2" t="s">
         <v>10</v>
@@ -4892,36 +5440,36 @@
         <v>16</v>
       </c>
       <c r="D6" s="2" t="s">
-        <v>206</v>
+        <v>202</v>
       </c>
       <c r="E6" s="2" t="b">
         <v>0</v>
       </c>
       <c r="F6" s="2" t="s">
-        <v>212</v>
+        <v>208</v>
       </c>
     </row>
     <row r="8" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A8" s="7" t="s">
+        <v>89</v>
+      </c>
+      <c r="B8" s="8" t="s">
+        <v>90</v>
+      </c>
+      <c r="C8" s="8" t="s">
+        <v>91</v>
+      </c>
+      <c r="D8" s="8" t="s">
+        <v>92</v>
+      </c>
+      <c r="E8" s="8" t="s">
         <v>93</v>
       </c>
-      <c r="B8" s="8" t="s">
+      <c r="F8" s="8" t="s">
         <v>94</v>
       </c>
-      <c r="C8" s="8" t="s">
-        <v>95</v>
-      </c>
-      <c r="D8" s="8" t="s">
-        <v>96</v>
-      </c>
-      <c r="E8" s="8" t="s">
-        <v>97</v>
-      </c>
-      <c r="F8" s="8" t="s">
-        <v>98</v>
-      </c>
       <c r="G8" s="9" t="s">
-        <v>83</v>
+        <v>79</v>
       </c>
     </row>
     <row r="9" spans="1:7" x14ac:dyDescent="0.3">
@@ -4929,22 +5477,22 @@
         <v>8</v>
       </c>
       <c r="B9" s="4" t="s">
-        <v>106</v>
+        <v>102</v>
       </c>
       <c r="C9" s="4" t="s">
-        <v>106</v>
+        <v>102</v>
       </c>
       <c r="D9" s="4" t="s">
-        <v>106</v>
+        <v>102</v>
       </c>
       <c r="E9" s="4" t="s">
-        <v>106</v>
+        <v>102</v>
       </c>
       <c r="F9" s="4" t="s">
-        <v>106</v>
+        <v>102</v>
       </c>
       <c r="G9" s="6" t="s">
-        <v>106</v>
+        <v>102</v>
       </c>
     </row>
     <row r="10" spans="1:7" x14ac:dyDescent="0.3">
@@ -4967,7 +5515,7 @@
         <v>43</v>
       </c>
       <c r="G10" s="6" t="s">
-        <v>209</v>
+        <v>205</v>
       </c>
     </row>
     <row r="11" spans="1:7" x14ac:dyDescent="0.3">
@@ -4990,7 +5538,7 @@
         <v>41</v>
       </c>
       <c r="G11" s="6" t="s">
-        <v>210</v>
+        <v>206</v>
       </c>
     </row>
     <row r="12" spans="1:7" x14ac:dyDescent="0.3">
@@ -5013,30 +5561,30 @@
         <v>47</v>
       </c>
       <c r="G12" s="6" t="s">
-        <v>211</v>
+        <v>207</v>
       </c>
     </row>
     <row r="13" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A13" s="10" t="s">
-        <v>205</v>
+        <v>201</v>
       </c>
       <c r="B13" s="11" t="s">
-        <v>205</v>
+        <v>201</v>
       </c>
       <c r="C13" s="11" t="s">
-        <v>205</v>
+        <v>201</v>
       </c>
       <c r="D13" s="11" t="s">
-        <v>207</v>
+        <v>203</v>
       </c>
       <c r="E13" s="11" t="s">
-        <v>205</v>
+        <v>201</v>
       </c>
       <c r="F13" s="11" t="s">
-        <v>106</v>
+        <v>102</v>
       </c>
       <c r="G13" s="12" t="s">
-        <v>106</v>
+        <v>102</v>
       </c>
     </row>
   </sheetData>
@@ -5068,7 +5616,7 @@
         <v>48</v>
       </c>
       <c r="D1" s="2" t="s">
-        <v>255</v>
+        <v>251</v>
       </c>
       <c r="E1" s="2" t="s">
         <v>7</v>
@@ -5107,7 +5655,7 @@
     </row>
     <row r="4" spans="1:5" ht="57.6" x14ac:dyDescent="0.3">
       <c r="A4" s="2" t="s">
-        <v>221</v>
+        <v>217</v>
       </c>
       <c r="B4" s="2" t="s">
         <v>10</v>
@@ -5119,12 +5667,12 @@
         <v>0</v>
       </c>
       <c r="E4" s="2" t="s">
-        <v>254</v>
+        <v>250</v>
       </c>
     </row>
     <row r="5" spans="1:5" ht="57.6" x14ac:dyDescent="0.3">
       <c r="A5" s="2" t="s">
-        <v>224</v>
+        <v>220</v>
       </c>
       <c r="B5" s="2" t="s">
         <v>10</v>
@@ -5136,12 +5684,12 @@
         <v>0</v>
       </c>
       <c r="E5" s="2" t="s">
-        <v>254</v>
+        <v>250</v>
       </c>
     </row>
     <row r="6" spans="1:5" ht="57.6" x14ac:dyDescent="0.3">
       <c r="A6" s="2" t="s">
-        <v>228</v>
+        <v>224</v>
       </c>
       <c r="B6" s="2" t="s">
         <v>10</v>
@@ -5153,12 +5701,12 @@
         <v>0</v>
       </c>
       <c r="E6" s="2" t="s">
-        <v>254</v>
+        <v>250</v>
       </c>
     </row>
     <row r="7" spans="1:5" ht="57.6" x14ac:dyDescent="0.3">
       <c r="A7" s="2" t="s">
-        <v>232</v>
+        <v>228</v>
       </c>
       <c r="B7" s="2" t="s">
         <v>10</v>
@@ -5170,12 +5718,12 @@
         <v>0</v>
       </c>
       <c r="E7" s="2" t="s">
-        <v>254</v>
+        <v>250</v>
       </c>
     </row>
     <row r="8" spans="1:5" ht="57.6" x14ac:dyDescent="0.3">
       <c r="A8" s="2" t="s">
-        <v>217</v>
+        <v>213</v>
       </c>
       <c r="B8" s="2" t="s">
         <v>10</v>
@@ -5187,12 +5735,12 @@
         <v>0</v>
       </c>
       <c r="E8" s="2" t="s">
-        <v>254</v>
+        <v>250</v>
       </c>
     </row>
     <row r="9" spans="1:5" ht="57.6" x14ac:dyDescent="0.3">
       <c r="A9" s="2" t="s">
-        <v>213</v>
+        <v>209</v>
       </c>
       <c r="B9" s="2" t="s">
         <v>10</v>
@@ -5204,12 +5752,12 @@
         <v>0</v>
       </c>
       <c r="E9" s="2" t="s">
-        <v>254</v>
+        <v>250</v>
       </c>
     </row>
     <row r="10" spans="1:5" ht="57.6" x14ac:dyDescent="0.3">
       <c r="A10" s="2" t="s">
-        <v>237</v>
+        <v>233</v>
       </c>
       <c r="B10" s="2" t="s">
         <v>10</v>
@@ -5221,12 +5769,12 @@
         <v>0</v>
       </c>
       <c r="E10" s="2" t="s">
-        <v>254</v>
+        <v>250</v>
       </c>
     </row>
     <row r="11" spans="1:5" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A11" s="2" t="s">
-        <v>241</v>
+        <v>237</v>
       </c>
       <c r="B11" s="2" t="s">
         <v>15</v>
@@ -5238,12 +5786,12 @@
         <v>0</v>
       </c>
       <c r="E11" s="2" t="s">
-        <v>257</v>
+        <v>253</v>
       </c>
     </row>
     <row r="12" spans="1:5" ht="57.6" x14ac:dyDescent="0.3">
       <c r="A12" s="2" t="s">
-        <v>247</v>
+        <v>243</v>
       </c>
       <c r="B12" s="2" t="s">
         <v>10</v>
@@ -5255,12 +5803,12 @@
         <v>0</v>
       </c>
       <c r="E12" s="2" t="s">
-        <v>254</v>
+        <v>250</v>
       </c>
     </row>
     <row r="13" spans="1:5" ht="57.6" x14ac:dyDescent="0.3">
       <c r="A13" s="2" t="s">
-        <v>251</v>
+        <v>247</v>
       </c>
       <c r="B13" s="2" t="s">
         <v>10</v>
@@ -5272,12 +5820,12 @@
         <v>1</v>
       </c>
       <c r="E13" s="2" t="s">
-        <v>256</v>
+        <v>252</v>
       </c>
     </row>
     <row r="14" spans="1:5" ht="57.6" x14ac:dyDescent="0.3">
       <c r="A14" s="2" t="s">
-        <v>252</v>
+        <v>248</v>
       </c>
       <c r="B14" s="2" t="s">
         <v>10</v>
@@ -5289,12 +5837,12 @@
         <v>1</v>
       </c>
       <c r="E14" s="2" t="s">
-        <v>256</v>
+        <v>252</v>
       </c>
     </row>
     <row r="15" spans="1:5" ht="57.6" x14ac:dyDescent="0.3">
       <c r="A15" s="2" t="s">
-        <v>253</v>
+        <v>249</v>
       </c>
       <c r="B15" s="2" t="s">
         <v>10</v>
@@ -5306,30 +5854,30 @@
         <v>1</v>
       </c>
       <c r="E15" s="2" t="s">
-        <v>256</v>
+        <v>252</v>
       </c>
     </row>
     <row r="17" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A17" s="7" t="s">
+        <v>89</v>
+      </c>
+      <c r="B17" s="8" t="s">
+        <v>90</v>
+      </c>
+      <c r="C17" s="8" t="s">
+        <v>91</v>
+      </c>
+      <c r="D17" s="8" t="s">
+        <v>92</v>
+      </c>
+      <c r="E17" s="8" t="s">
         <v>93</v>
       </c>
-      <c r="B17" s="8" t="s">
+      <c r="F17" s="8" t="s">
         <v>94</v>
       </c>
-      <c r="C17" s="8" t="s">
-        <v>95</v>
-      </c>
-      <c r="D17" s="8" t="s">
-        <v>96</v>
-      </c>
-      <c r="E17" s="8" t="s">
-        <v>97</v>
-      </c>
-      <c r="F17" s="8" t="s">
-        <v>98</v>
-      </c>
       <c r="G17" s="9" t="s">
-        <v>83</v>
+        <v>79</v>
       </c>
     </row>
     <row r="18" spans="1:7" x14ac:dyDescent="0.3">
@@ -5375,24 +5923,24 @@
         <v>43</v>
       </c>
       <c r="G19" s="6" t="s">
-        <v>209</v>
+        <v>205</v>
       </c>
     </row>
     <row r="20" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A20" s="5" t="s">
-        <v>213</v>
+        <v>209</v>
       </c>
       <c r="B20" s="4" t="s">
-        <v>214</v>
+        <v>210</v>
       </c>
       <c r="C20" s="4" t="s">
-        <v>214</v>
+        <v>210</v>
       </c>
       <c r="D20" s="4" t="s">
-        <v>215</v>
+        <v>211</v>
       </c>
       <c r="E20" s="4" t="s">
-        <v>216</v>
+        <v>212</v>
       </c>
       <c r="F20" s="4" t="s">
         <v>9</v>
@@ -5403,68 +5951,68 @@
     </row>
     <row r="21" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A21" s="5" t="s">
-        <v>217</v>
+        <v>213</v>
       </c>
       <c r="B21" s="4" t="s">
-        <v>217</v>
+        <v>213</v>
       </c>
       <c r="C21" s="4" t="s">
-        <v>217</v>
+        <v>213</v>
       </c>
       <c r="D21" s="4" t="s">
-        <v>218</v>
+        <v>214</v>
       </c>
       <c r="E21" s="4" t="s">
-        <v>217</v>
+        <v>213</v>
       </c>
       <c r="F21" s="4" t="s">
-        <v>219</v>
+        <v>215</v>
       </c>
       <c r="G21" s="6" t="s">
-        <v>220</v>
+        <v>216</v>
       </c>
     </row>
     <row r="22" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A22" s="5" t="s">
-        <v>221</v>
+        <v>217</v>
       </c>
       <c r="B22" s="4" t="s">
-        <v>221</v>
+        <v>217</v>
       </c>
       <c r="C22" s="4" t="s">
-        <v>221</v>
+        <v>217</v>
       </c>
       <c r="D22" s="4" t="s">
-        <v>222</v>
+        <v>218</v>
       </c>
       <c r="E22" s="4" t="s">
-        <v>221</v>
+        <v>217</v>
       </c>
       <c r="F22" s="4" t="s">
-        <v>222</v>
+        <v>218</v>
       </c>
       <c r="G22" s="6" t="s">
-        <v>223</v>
+        <v>219</v>
       </c>
     </row>
     <row r="23" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A23" s="5" t="s">
-        <v>224</v>
+        <v>220</v>
       </c>
       <c r="B23" s="4" t="s">
-        <v>224</v>
+        <v>220</v>
       </c>
       <c r="C23" s="4" t="s">
-        <v>224</v>
+        <v>220</v>
       </c>
       <c r="D23" s="4" t="s">
-        <v>225</v>
+        <v>221</v>
       </c>
       <c r="E23" s="4" t="s">
-        <v>226</v>
+        <v>222</v>
       </c>
       <c r="F23" s="4" t="s">
-        <v>227</v>
+        <v>223</v>
       </c>
       <c r="G23" s="6" t="s">
         <v>9</v>
@@ -5472,45 +6020,45 @@
     </row>
     <row r="24" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A24" s="5" t="s">
-        <v>228</v>
+        <v>224</v>
       </c>
       <c r="B24" s="4" t="s">
-        <v>228</v>
+        <v>224</v>
       </c>
       <c r="C24" s="4" t="s">
-        <v>228</v>
+        <v>224</v>
       </c>
       <c r="D24" s="4" t="s">
-        <v>229</v>
+        <v>225</v>
       </c>
       <c r="E24" s="4" t="s">
-        <v>230</v>
+        <v>226</v>
       </c>
       <c r="F24" s="4" t="s">
         <v>9</v>
       </c>
       <c r="G24" s="6" t="s">
-        <v>231</v>
+        <v>227</v>
       </c>
     </row>
     <row r="25" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A25" s="5" t="s">
+        <v>228</v>
+      </c>
+      <c r="B25" s="4" t="s">
+        <v>229</v>
+      </c>
+      <c r="C25" s="4" t="s">
+        <v>229</v>
+      </c>
+      <c r="D25" s="4" t="s">
+        <v>230</v>
+      </c>
+      <c r="E25" s="4" t="s">
+        <v>231</v>
+      </c>
+      <c r="F25" s="4" t="s">
         <v>232</v>
-      </c>
-      <c r="B25" s="4" t="s">
-        <v>233</v>
-      </c>
-      <c r="C25" s="4" t="s">
-        <v>233</v>
-      </c>
-      <c r="D25" s="4" t="s">
-        <v>234</v>
-      </c>
-      <c r="E25" s="4" t="s">
-        <v>235</v>
-      </c>
-      <c r="F25" s="4" t="s">
-        <v>236</v>
       </c>
       <c r="G25" s="6" t="s">
         <v>9</v>
@@ -5518,76 +6066,76 @@
     </row>
     <row r="26" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A26" s="5" t="s">
-        <v>237</v>
+        <v>233</v>
       </c>
       <c r="B26" s="4" t="s">
-        <v>237</v>
+        <v>233</v>
       </c>
       <c r="C26" s="4" t="s">
-        <v>237</v>
+        <v>233</v>
       </c>
       <c r="D26" s="4" t="s">
-        <v>238</v>
+        <v>234</v>
       </c>
       <c r="E26" s="4" t="s">
-        <v>237</v>
+        <v>233</v>
       </c>
       <c r="F26" s="4" t="s">
-        <v>239</v>
+        <v>235</v>
       </c>
       <c r="G26" s="6" t="s">
-        <v>240</v>
+        <v>236</v>
       </c>
     </row>
     <row r="27" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A27" s="5" t="s">
+        <v>237</v>
+      </c>
+      <c r="B27" s="4" t="s">
+        <v>238</v>
+      </c>
+      <c r="C27" s="4" t="s">
+        <v>238</v>
+      </c>
+      <c r="D27" s="4" t="s">
+        <v>239</v>
+      </c>
+      <c r="E27" s="4" t="s">
+        <v>240</v>
+      </c>
+      <c r="F27" s="4" t="s">
         <v>241</v>
       </c>
-      <c r="B27" s="4" t="s">
+      <c r="G27" s="6" t="s">
         <v>242</v>
-      </c>
-      <c r="C27" s="4" t="s">
-        <v>242</v>
-      </c>
-      <c r="D27" s="4" t="s">
-        <v>243</v>
-      </c>
-      <c r="E27" s="4" t="s">
-        <v>244</v>
-      </c>
-      <c r="F27" s="4" t="s">
-        <v>245</v>
-      </c>
-      <c r="G27" s="6" t="s">
-        <v>246</v>
       </c>
     </row>
     <row r="28" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A28" s="5" t="s">
-        <v>247</v>
+        <v>243</v>
       </c>
       <c r="B28" s="4" t="s">
-        <v>248</v>
+        <v>244</v>
       </c>
       <c r="C28" s="4" t="s">
-        <v>248</v>
+        <v>244</v>
       </c>
       <c r="D28" s="4" t="s">
-        <v>249</v>
+        <v>245</v>
       </c>
       <c r="E28" s="4" t="s">
-        <v>247</v>
+        <v>243</v>
       </c>
       <c r="F28" s="4" t="s">
-        <v>249</v>
+        <v>245</v>
       </c>
       <c r="G28" s="6" t="s">
-        <v>250</v>
+        <v>246</v>
       </c>
     </row>
     <row r="29" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A29" s="5" t="s">
-        <v>251</v>
+        <v>247</v>
       </c>
       <c r="B29" s="4" t="s">
         <v>9</v>
@@ -5610,7 +6158,7 @@
     </row>
     <row r="30" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A30" s="5" t="s">
-        <v>252</v>
+        <v>248</v>
       </c>
       <c r="B30" s="4" t="s">
         <v>9</v>
@@ -5633,7 +6181,7 @@
     </row>
     <row r="31" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A31" s="10" t="s">
-        <v>253</v>
+        <v>249</v>
       </c>
       <c r="B31" s="11" t="s">
         <v>9</v>
@@ -5675,178 +6223,178 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:8" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A1" s="15" t="s">
+      <c r="A1" s="14" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="15" t="s">
+      <c r="B1" s="14" t="s">
         <v>48</v>
       </c>
-      <c r="C1" s="15" t="s">
+      <c r="C1" s="14" t="s">
         <v>49</v>
       </c>
-      <c r="D1" s="15" t="s">
+      <c r="D1" s="14" t="s">
         <v>7</v>
       </c>
     </row>
     <row r="2" spans="1:8" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="A2" s="16" t="s">
+      <c r="A2" s="15" t="s">
         <v>8</v>
       </c>
-      <c r="B2" s="16" t="s">
+      <c r="B2" s="15" t="s">
         <v>10</v>
       </c>
-      <c r="C2" s="16" t="b">
+      <c r="C2" s="15" t="b">
         <v>0</v>
       </c>
-      <c r="D2" s="16" t="s">
+      <c r="D2" s="15" t="s">
         <v>12</v>
       </c>
     </row>
     <row r="3" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A3" s="17" t="s">
+      <c r="A3" s="16" t="s">
         <v>29</v>
       </c>
-      <c r="B3" s="17" t="s">
+      <c r="B3" s="16" t="s">
         <v>18</v>
       </c>
-      <c r="C3" s="17" t="b">
+      <c r="C3" s="16" t="b">
         <v>0</v>
       </c>
-      <c r="D3" s="17"/>
+      <c r="D3" s="16"/>
     </row>
     <row r="4" spans="1:8" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="A4" s="16" t="s">
+      <c r="A4" s="15" t="s">
         <v>50</v>
       </c>
-      <c r="B4" s="16" t="s">
+      <c r="B4" s="15" t="s">
         <v>10</v>
       </c>
-      <c r="C4" s="16" t="b">
+      <c r="C4" s="15" t="b">
         <v>1</v>
       </c>
-      <c r="D4" s="16" t="s">
-        <v>265</v>
+      <c r="D4" s="15" t="s">
+        <v>261</v>
       </c>
     </row>
     <row r="5" spans="1:8" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="A5" s="17" t="s">
+      <c r="A5" s="16" t="s">
         <v>51</v>
       </c>
-      <c r="B5" s="17" t="s">
+      <c r="B5" s="16" t="s">
         <v>15</v>
       </c>
-      <c r="C5" s="17" t="b">
+      <c r="C5" s="16" t="b">
         <v>1</v>
       </c>
-      <c r="D5" s="17" t="s">
-        <v>265</v>
+      <c r="D5" s="16" t="s">
+        <v>261</v>
       </c>
     </row>
     <row r="6" spans="1:8" ht="43.2" x14ac:dyDescent="0.3">
-      <c r="A6" s="16" t="s">
+      <c r="A6" s="15" t="s">
         <v>56</v>
       </c>
-      <c r="B6" s="16" t="s">
+      <c r="B6" s="15" t="s">
         <v>15</v>
       </c>
-      <c r="C6" s="16" t="b">
+      <c r="C6" s="15" t="b">
         <v>1</v>
       </c>
-      <c r="D6" s="16" t="s">
+      <c r="D6" s="15" t="s">
         <v>57</v>
       </c>
     </row>
     <row r="7" spans="1:8" ht="57.6" x14ac:dyDescent="0.3">
-      <c r="A7" s="17" t="s">
+      <c r="A7" s="16" t="s">
         <v>58</v>
       </c>
-      <c r="B7" s="17" t="s">
+      <c r="B7" s="16" t="s">
         <v>10</v>
       </c>
-      <c r="C7" s="17" t="b">
+      <c r="C7" s="16" t="b">
         <v>1</v>
       </c>
-      <c r="D7" s="17" t="s">
+      <c r="D7" s="16" t="s">
         <v>59</v>
       </c>
     </row>
     <row r="8" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A8" s="16" t="s">
+      <c r="A8" s="15" t="s">
         <v>52</v>
       </c>
-      <c r="B8" s="16" t="s">
+      <c r="B8" s="15" t="s">
         <v>10</v>
       </c>
-      <c r="C8" s="16" t="s">
-        <v>9</v>
-      </c>
-      <c r="D8" s="16" t="s">
+      <c r="C8" s="15" t="s">
+        <v>9</v>
+      </c>
+      <c r="D8" s="15" t="s">
         <v>9</v>
       </c>
     </row>
     <row r="9" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A9" s="17" t="s">
+      <c r="A9" s="16" t="s">
         <v>53</v>
       </c>
-      <c r="B9" s="17" t="s">
+      <c r="B9" s="16" t="s">
         <v>15</v>
       </c>
-      <c r="C9" s="17" t="s">
-        <v>9</v>
-      </c>
-      <c r="D9" s="17" t="s">
+      <c r="C9" s="16" t="s">
+        <v>9</v>
+      </c>
+      <c r="D9" s="16" t="s">
         <v>9</v>
       </c>
     </row>
     <row r="10" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A10" s="16" t="s">
+      <c r="A10" s="15" t="s">
         <v>54</v>
       </c>
-      <c r="B10" s="16" t="s">
+      <c r="B10" s="15" t="s">
         <v>15</v>
       </c>
-      <c r="C10" s="16" t="s">
-        <v>9</v>
-      </c>
-      <c r="D10" s="16" t="s">
+      <c r="C10" s="15" t="s">
+        <v>9</v>
+      </c>
+      <c r="D10" s="15" t="s">
         <v>9</v>
       </c>
     </row>
     <row r="11" spans="1:8" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A11" s="18" t="s">
+      <c r="A11" s="17" t="s">
         <v>54</v>
       </c>
-      <c r="B11" s="18" t="s">
+      <c r="B11" s="17" t="s">
         <v>15</v>
       </c>
-      <c r="C11" s="18" t="s">
-        <v>9</v>
-      </c>
-      <c r="D11" s="18" t="s">
+      <c r="C11" s="17" t="s">
+        <v>9</v>
+      </c>
+      <c r="D11" s="17" t="s">
         <v>9</v>
       </c>
     </row>
     <row r="13" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A13" s="7" t="s">
+        <v>89</v>
+      </c>
+      <c r="B13" s="8" t="s">
+        <v>90</v>
+      </c>
+      <c r="C13" s="8" t="s">
+        <v>91</v>
+      </c>
+      <c r="D13" s="8" t="s">
+        <v>92</v>
+      </c>
+      <c r="E13" s="8" t="s">
         <v>93</v>
       </c>
-      <c r="B13" s="8" t="s">
+      <c r="F13" s="8" t="s">
         <v>94</v>
       </c>
-      <c r="C13" s="8" t="s">
-        <v>95</v>
-      </c>
-      <c r="D13" s="8" t="s">
-        <v>96</v>
-      </c>
-      <c r="E13" s="8" t="s">
-        <v>97</v>
-      </c>
-      <c r="F13" s="8" t="s">
-        <v>98</v>
-      </c>
       <c r="G13" s="9" t="s">
-        <v>83</v>
+        <v>79</v>
       </c>
       <c r="H13" s="8" t="s">
         <v>7</v>
@@ -5854,25 +6402,25 @@
     </row>
     <row r="14" spans="1:8" ht="41.4" x14ac:dyDescent="0.3">
       <c r="A14" s="5" t="s">
-        <v>258</v>
+        <v>254</v>
       </c>
       <c r="B14" s="4" t="s">
-        <v>258</v>
+        <v>254</v>
       </c>
       <c r="C14" s="4" t="s">
-        <v>258</v>
+        <v>254</v>
       </c>
       <c r="D14" s="4" t="s">
-        <v>259</v>
+        <v>255</v>
       </c>
       <c r="E14" s="4" t="s">
-        <v>258</v>
+        <v>254</v>
       </c>
       <c r="F14" s="4" t="s">
-        <v>260</v>
+        <v>256</v>
       </c>
       <c r="G14" s="6" t="s">
-        <v>261</v>
+        <v>257</v>
       </c>
       <c r="H14" s="13" t="s">
         <v>63</v>
@@ -5880,25 +6428,25 @@
     </row>
     <row r="15" spans="1:8" ht="41.4" x14ac:dyDescent="0.3">
       <c r="A15" s="10" t="s">
-        <v>262</v>
+        <v>258</v>
       </c>
       <c r="B15" s="11" t="s">
-        <v>262</v>
+        <v>258</v>
       </c>
       <c r="C15" s="11" t="s">
-        <v>262</v>
+        <v>258</v>
       </c>
       <c r="D15" s="11" t="s">
-        <v>263</v>
+        <v>259</v>
       </c>
       <c r="E15" s="11" t="s">
-        <v>262</v>
+        <v>258</v>
       </c>
       <c r="F15" s="11" t="s">
-        <v>264</v>
+        <v>260</v>
       </c>
       <c r="G15" s="12" t="s">
-        <v>106</v>
+        <v>102</v>
       </c>
       <c r="H15" s="11" t="s">
         <v>63</v>
@@ -5969,6 +6517,1078 @@
       <c r="B29" s="2"/>
       <c r="C29" s="2"/>
       <c r="D29" s="2"/>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <tableParts count="1">
+    <tablePart r:id="rId1"/>
+  </tableParts>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B560DDC0-B460-478C-A8D1-D2C3187C3DD6}">
+  <dimension ref="A1:G62"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="1" max="4" width="19.77734375" style="2" customWidth="1"/>
+    <col min="5" max="5" width="87.6640625" style="2" customWidth="1"/>
+    <col min="6" max="16384" width="8.88671875" style="2"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A1" s="20" t="s">
+        <v>262</v>
+      </c>
+      <c r="B1" s="20" t="s">
+        <v>263</v>
+      </c>
+      <c r="C1" s="20" t="s">
+        <v>264</v>
+      </c>
+      <c r="D1" s="20" t="s">
+        <v>265</v>
+      </c>
+      <c r="E1" s="20" t="s">
+        <v>266</v>
+      </c>
+    </row>
+    <row r="2" spans="1:5" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A2" s="18" t="s">
+        <v>29</v>
+      </c>
+      <c r="B2" s="18" t="s">
+        <v>272</v>
+      </c>
+      <c r="C2" s="18" t="s">
+        <v>273</v>
+      </c>
+      <c r="D2" s="18" t="s">
+        <v>274</v>
+      </c>
+      <c r="E2" s="18" t="s">
+        <v>275</v>
+      </c>
+    </row>
+    <row r="3" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A3" s="18" t="s">
+        <v>8</v>
+      </c>
+      <c r="B3" s="18" t="s">
+        <v>267</v>
+      </c>
+      <c r="C3" s="18" t="s">
+        <v>9</v>
+      </c>
+      <c r="D3" s="18" t="s">
+        <v>268</v>
+      </c>
+      <c r="E3" s="18" t="s">
+        <v>269</v>
+      </c>
+    </row>
+    <row r="4" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A4" s="18" t="s">
+        <v>95</v>
+      </c>
+      <c r="B4" s="18" t="s">
+        <v>281</v>
+      </c>
+      <c r="C4" s="18" t="s">
+        <v>313</v>
+      </c>
+      <c r="D4" s="18" t="s">
+        <v>314</v>
+      </c>
+      <c r="E4" s="18" t="s">
+        <v>315</v>
+      </c>
+    </row>
+    <row r="5" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A5" s="18" t="s">
+        <v>100</v>
+      </c>
+      <c r="B5" s="18" t="s">
+        <v>281</v>
+      </c>
+      <c r="C5" s="18" t="s">
+        <v>313</v>
+      </c>
+      <c r="D5" s="18" t="s">
+        <v>314</v>
+      </c>
+      <c r="E5" s="18" t="s">
+        <v>316</v>
+      </c>
+    </row>
+    <row r="6" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A6" s="18" t="s">
+        <v>103</v>
+      </c>
+      <c r="B6" s="18" t="s">
+        <v>281</v>
+      </c>
+      <c r="C6" s="18" t="s">
+        <v>313</v>
+      </c>
+      <c r="D6" s="18" t="s">
+        <v>314</v>
+      </c>
+      <c r="E6" s="18" t="s">
+        <v>317</v>
+      </c>
+    </row>
+    <row r="7" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A7" s="18" t="s">
+        <v>108</v>
+      </c>
+      <c r="B7" s="18" t="s">
+        <v>281</v>
+      </c>
+      <c r="C7" s="18" t="s">
+        <v>318</v>
+      </c>
+      <c r="D7" s="18" t="s">
+        <v>314</v>
+      </c>
+      <c r="E7" s="18" t="s">
+        <v>319</v>
+      </c>
+    </row>
+    <row r="8" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A8" s="18" t="s">
+        <v>112</v>
+      </c>
+      <c r="B8" s="18" t="s">
+        <v>281</v>
+      </c>
+      <c r="C8" s="18" t="s">
+        <v>318</v>
+      </c>
+      <c r="D8" s="18" t="s">
+        <v>314</v>
+      </c>
+      <c r="E8" s="18" t="s">
+        <v>320</v>
+      </c>
+    </row>
+    <row r="9" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A9" s="18" t="s">
+        <v>116</v>
+      </c>
+      <c r="B9" s="18" t="s">
+        <v>281</v>
+      </c>
+      <c r="C9" s="18" t="s">
+        <v>318</v>
+      </c>
+      <c r="D9" s="18" t="s">
+        <v>314</v>
+      </c>
+      <c r="E9" s="18" t="s">
+        <v>321</v>
+      </c>
+    </row>
+    <row r="10" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A10" s="18" t="s">
+        <v>119</v>
+      </c>
+      <c r="B10" s="18" t="s">
+        <v>281</v>
+      </c>
+      <c r="C10" s="18" t="s">
+        <v>313</v>
+      </c>
+      <c r="D10" s="18" t="s">
+        <v>314</v>
+      </c>
+      <c r="E10" s="18" t="s">
+        <v>322</v>
+      </c>
+    </row>
+    <row r="11" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A11" s="18" t="s">
+        <v>124</v>
+      </c>
+      <c r="B11" s="18" t="s">
+        <v>281</v>
+      </c>
+      <c r="C11" s="18" t="s">
+        <v>313</v>
+      </c>
+      <c r="D11" s="18" t="s">
+        <v>314</v>
+      </c>
+      <c r="E11" s="18" t="s">
+        <v>323</v>
+      </c>
+    </row>
+    <row r="12" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A12" s="18" t="s">
+        <v>127</v>
+      </c>
+      <c r="B12" s="18" t="s">
+        <v>281</v>
+      </c>
+      <c r="C12" s="18" t="s">
+        <v>318</v>
+      </c>
+      <c r="D12" s="18" t="s">
+        <v>314</v>
+      </c>
+      <c r="E12" s="18" t="s">
+        <v>324</v>
+      </c>
+    </row>
+    <row r="13" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A13" s="18" t="s">
+        <v>131</v>
+      </c>
+      <c r="B13" s="18" t="s">
+        <v>281</v>
+      </c>
+      <c r="C13" s="18" t="s">
+        <v>325</v>
+      </c>
+      <c r="D13" s="18" t="s">
+        <v>314</v>
+      </c>
+      <c r="E13" s="18" t="s">
+        <v>326</v>
+      </c>
+    </row>
+    <row r="14" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A14" s="18" t="s">
+        <v>136</v>
+      </c>
+      <c r="B14" s="18" t="s">
+        <v>281</v>
+      </c>
+      <c r="C14" s="18" t="s">
+        <v>325</v>
+      </c>
+      <c r="D14" s="18" t="s">
+        <v>314</v>
+      </c>
+      <c r="E14" s="18" t="s">
+        <v>327</v>
+      </c>
+    </row>
+    <row r="15" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A15" s="18" t="s">
+        <v>139</v>
+      </c>
+      <c r="B15" s="18" t="s">
+        <v>281</v>
+      </c>
+      <c r="C15" s="18" t="s">
+        <v>328</v>
+      </c>
+      <c r="D15" s="18" t="s">
+        <v>314</v>
+      </c>
+      <c r="E15" s="18" t="s">
+        <v>329</v>
+      </c>
+    </row>
+    <row r="16" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A16" s="18" t="s">
+        <v>143</v>
+      </c>
+      <c r="B16" s="18" t="s">
+        <v>281</v>
+      </c>
+      <c r="C16" s="18" t="s">
+        <v>330</v>
+      </c>
+      <c r="D16" s="18" t="s">
+        <v>314</v>
+      </c>
+      <c r="E16" s="18" t="s">
+        <v>331</v>
+      </c>
+    </row>
+    <row r="17" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A17" s="18" t="s">
+        <v>148</v>
+      </c>
+      <c r="B17" s="18" t="s">
+        <v>281</v>
+      </c>
+      <c r="C17" s="18" t="s">
+        <v>332</v>
+      </c>
+      <c r="D17" s="18" t="s">
+        <v>314</v>
+      </c>
+      <c r="E17" s="18" t="s">
+        <v>333</v>
+      </c>
+    </row>
+    <row r="18" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A18" s="18" t="s">
+        <v>152</v>
+      </c>
+      <c r="B18" s="18" t="s">
+        <v>281</v>
+      </c>
+      <c r="C18" s="18" t="s">
+        <v>328</v>
+      </c>
+      <c r="D18" s="18" t="s">
+        <v>314</v>
+      </c>
+      <c r="E18" s="18" t="s">
+        <v>334</v>
+      </c>
+    </row>
+    <row r="19" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A19" s="18" t="s">
+        <v>156</v>
+      </c>
+      <c r="B19" s="18" t="s">
+        <v>281</v>
+      </c>
+      <c r="C19" s="18" t="s">
+        <v>9</v>
+      </c>
+      <c r="D19" s="18" t="s">
+        <v>314</v>
+      </c>
+      <c r="E19" s="18" t="s">
+        <v>335</v>
+      </c>
+    </row>
+    <row r="20" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A20" s="18" t="s">
+        <v>160</v>
+      </c>
+      <c r="B20" s="18" t="s">
+        <v>281</v>
+      </c>
+      <c r="C20" s="18" t="s">
+        <v>313</v>
+      </c>
+      <c r="D20" s="18" t="s">
+        <v>314</v>
+      </c>
+      <c r="E20" s="18" t="s">
+        <v>336</v>
+      </c>
+    </row>
+    <row r="21" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A21" s="18" t="s">
+        <v>165</v>
+      </c>
+      <c r="B21" s="18" t="s">
+        <v>281</v>
+      </c>
+      <c r="C21" s="18" t="s">
+        <v>313</v>
+      </c>
+      <c r="D21" s="18" t="s">
+        <v>314</v>
+      </c>
+      <c r="E21" s="18" t="s">
+        <v>337</v>
+      </c>
+    </row>
+    <row r="22" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A22" s="18" t="s">
+        <v>169</v>
+      </c>
+      <c r="B22" s="18" t="s">
+        <v>281</v>
+      </c>
+      <c r="C22" s="18" t="s">
+        <v>313</v>
+      </c>
+      <c r="D22" s="18" t="s">
+        <v>314</v>
+      </c>
+      <c r="E22" s="18" t="s">
+        <v>338</v>
+      </c>
+    </row>
+    <row r="23" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A23" s="18" t="s">
+        <v>173</v>
+      </c>
+      <c r="B23" s="18" t="s">
+        <v>281</v>
+      </c>
+      <c r="C23" s="18" t="s">
+        <v>313</v>
+      </c>
+      <c r="D23" s="18" t="s">
+        <v>314</v>
+      </c>
+      <c r="E23" s="18" t="s">
+        <v>339</v>
+      </c>
+    </row>
+    <row r="24" spans="1:5" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A24" s="18" t="s">
+        <v>193</v>
+      </c>
+      <c r="B24" s="18" t="s">
+        <v>16</v>
+      </c>
+      <c r="C24" s="18" t="s">
+        <v>340</v>
+      </c>
+      <c r="D24" s="18" t="s">
+        <v>314</v>
+      </c>
+      <c r="E24" s="18" t="s">
+        <v>341</v>
+      </c>
+    </row>
+    <row r="25" spans="1:5" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A25" s="18" t="s">
+        <v>188</v>
+      </c>
+      <c r="B25" s="18" t="s">
+        <v>16</v>
+      </c>
+      <c r="C25" s="18" t="s">
+        <v>340</v>
+      </c>
+      <c r="D25" s="18" t="s">
+        <v>314</v>
+      </c>
+      <c r="E25" s="18" t="s">
+        <v>342</v>
+      </c>
+    </row>
+    <row r="26" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A26" s="18" t="s">
+        <v>178</v>
+      </c>
+      <c r="B26" s="18" t="s">
+        <v>281</v>
+      </c>
+      <c r="C26" s="18" t="s">
+        <v>328</v>
+      </c>
+      <c r="D26" s="18" t="s">
+        <v>314</v>
+      </c>
+      <c r="E26" s="18" t="s">
+        <v>344</v>
+      </c>
+    </row>
+    <row r="27" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A27" s="18" t="s">
+        <v>183</v>
+      </c>
+      <c r="B27" s="18" t="s">
+        <v>281</v>
+      </c>
+      <c r="C27" s="18" t="s">
+        <v>330</v>
+      </c>
+      <c r="D27" s="18" t="s">
+        <v>314</v>
+      </c>
+      <c r="E27" s="18" t="s">
+        <v>345</v>
+      </c>
+    </row>
+    <row r="28" spans="1:5" ht="86.4" x14ac:dyDescent="0.3">
+      <c r="A28" s="18" t="s">
+        <v>201</v>
+      </c>
+      <c r="B28" s="18" t="s">
+        <v>16</v>
+      </c>
+      <c r="C28" s="18" t="s">
+        <v>285</v>
+      </c>
+      <c r="D28" s="18" t="s">
+        <v>286</v>
+      </c>
+      <c r="E28" s="18" t="s">
+        <v>287</v>
+      </c>
+    </row>
+    <row r="29" spans="1:5" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A29" s="18" t="s">
+        <v>27</v>
+      </c>
+      <c r="B29" s="18" t="s">
+        <v>281</v>
+      </c>
+      <c r="C29" s="18" t="s">
+        <v>282</v>
+      </c>
+      <c r="D29" s="18" t="s">
+        <v>283</v>
+      </c>
+      <c r="E29" s="18" t="s">
+        <v>284</v>
+      </c>
+    </row>
+    <row r="30" spans="1:5" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A30" s="18" t="s">
+        <v>13</v>
+      </c>
+      <c r="B30" s="18" t="s">
+        <v>16</v>
+      </c>
+      <c r="C30" s="18" t="s">
+        <v>288</v>
+      </c>
+      <c r="D30" s="18" t="s">
+        <v>283</v>
+      </c>
+      <c r="E30" s="18" t="s">
+        <v>289</v>
+      </c>
+    </row>
+    <row r="31" spans="1:5" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A31" s="18" t="s">
+        <v>306</v>
+      </c>
+      <c r="B31" s="18" t="s">
+        <v>16</v>
+      </c>
+      <c r="C31" s="18" t="s">
+        <v>307</v>
+      </c>
+      <c r="D31" s="18" t="s">
+        <v>257</v>
+      </c>
+      <c r="E31" s="18" t="s">
+        <v>308</v>
+      </c>
+    </row>
+    <row r="32" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A32" s="18" t="s">
+        <v>254</v>
+      </c>
+      <c r="B32" s="18" t="s">
+        <v>281</v>
+      </c>
+      <c r="C32" s="18" t="s">
+        <v>309</v>
+      </c>
+      <c r="D32" s="18" t="s">
+        <v>257</v>
+      </c>
+      <c r="E32" s="18" t="s">
+        <v>310</v>
+      </c>
+    </row>
+    <row r="33" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A33" s="18" t="s">
+        <v>258</v>
+      </c>
+      <c r="B33" s="18" t="s">
+        <v>281</v>
+      </c>
+      <c r="C33" s="18" t="s">
+        <v>311</v>
+      </c>
+      <c r="D33" s="18" t="s">
+        <v>257</v>
+      </c>
+      <c r="E33" s="18" t="s">
+        <v>312</v>
+      </c>
+    </row>
+    <row r="34" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A34" s="18" t="s">
+        <v>217</v>
+      </c>
+      <c r="B34" s="18" t="s">
+        <v>16</v>
+      </c>
+      <c r="C34" s="18" t="s">
+        <v>290</v>
+      </c>
+      <c r="D34" s="18" t="s">
+        <v>291</v>
+      </c>
+      <c r="E34" s="18" t="s">
+        <v>292</v>
+      </c>
+    </row>
+    <row r="35" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A35" s="18" t="s">
+        <v>220</v>
+      </c>
+      <c r="B35" s="18" t="s">
+        <v>16</v>
+      </c>
+      <c r="C35" s="18" t="s">
+        <v>290</v>
+      </c>
+      <c r="D35" s="18" t="s">
+        <v>291</v>
+      </c>
+      <c r="E35" s="18" t="s">
+        <v>293</v>
+      </c>
+    </row>
+    <row r="36" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A36" s="18" t="s">
+        <v>224</v>
+      </c>
+      <c r="B36" s="18" t="s">
+        <v>16</v>
+      </c>
+      <c r="C36" s="18" t="s">
+        <v>290</v>
+      </c>
+      <c r="D36" s="18" t="s">
+        <v>291</v>
+      </c>
+      <c r="E36" s="18" t="s">
+        <v>294</v>
+      </c>
+    </row>
+    <row r="37" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A37" s="18" t="s">
+        <v>228</v>
+      </c>
+      <c r="B37" s="18" t="s">
+        <v>16</v>
+      </c>
+      <c r="C37" s="18" t="s">
+        <v>290</v>
+      </c>
+      <c r="D37" s="18" t="s">
+        <v>291</v>
+      </c>
+      <c r="E37" s="18" t="s">
+        <v>295</v>
+      </c>
+    </row>
+    <row r="38" spans="1:7" ht="43.2" x14ac:dyDescent="0.3">
+      <c r="A38" s="18" t="s">
+        <v>213</v>
+      </c>
+      <c r="B38" s="18" t="s">
+        <v>16</v>
+      </c>
+      <c r="C38" s="18" t="s">
+        <v>296</v>
+      </c>
+      <c r="D38" s="18" t="s">
+        <v>291</v>
+      </c>
+      <c r="E38" s="18" t="s">
+        <v>297</v>
+      </c>
+    </row>
+    <row r="39" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A39" s="18" t="s">
+        <v>209</v>
+      </c>
+      <c r="B39" s="18" t="s">
+        <v>16</v>
+      </c>
+      <c r="C39" s="18" t="s">
+        <v>290</v>
+      </c>
+      <c r="D39" s="18" t="s">
+        <v>291</v>
+      </c>
+      <c r="E39" s="18" t="s">
+        <v>343</v>
+      </c>
+    </row>
+    <row r="40" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A40" s="18" t="s">
+        <v>247</v>
+      </c>
+      <c r="B40" s="18" t="s">
+        <v>16</v>
+      </c>
+      <c r="C40" s="18"/>
+      <c r="D40" s="18" t="s">
+        <v>291</v>
+      </c>
+      <c r="E40" s="18" t="s">
+        <v>348</v>
+      </c>
+    </row>
+    <row r="41" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A41" s="18" t="s">
+        <v>249</v>
+      </c>
+      <c r="B41" s="18" t="s">
+        <v>16</v>
+      </c>
+      <c r="C41" s="18"/>
+      <c r="D41" s="18" t="s">
+        <v>291</v>
+      </c>
+      <c r="E41" s="18" t="s">
+        <v>347</v>
+      </c>
+    </row>
+    <row r="42" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A42" s="18" t="s">
+        <v>237</v>
+      </c>
+      <c r="B42" s="18" t="s">
+        <v>281</v>
+      </c>
+      <c r="C42" s="18" t="s">
+        <v>350</v>
+      </c>
+      <c r="D42" s="18" t="s">
+        <v>291</v>
+      </c>
+      <c r="E42" s="18" t="s">
+        <v>357</v>
+      </c>
+    </row>
+    <row r="43" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A43" s="18" t="s">
+        <v>243</v>
+      </c>
+      <c r="B43" s="18" t="s">
+        <v>16</v>
+      </c>
+      <c r="C43" s="18" t="s">
+        <v>290</v>
+      </c>
+      <c r="D43" s="18" t="s">
+        <v>291</v>
+      </c>
+      <c r="E43" s="18" t="s">
+        <v>354</v>
+      </c>
+    </row>
+    <row r="44" spans="1:7" ht="43.2" x14ac:dyDescent="0.3">
+      <c r="A44" s="18" t="s">
+        <v>233</v>
+      </c>
+      <c r="B44" s="18" t="s">
+        <v>16</v>
+      </c>
+      <c r="C44" s="18" t="s">
+        <v>360</v>
+      </c>
+      <c r="D44" s="18" t="s">
+        <v>291</v>
+      </c>
+      <c r="E44" s="18" t="s">
+        <v>359</v>
+      </c>
+    </row>
+    <row r="45" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A45" s="18" t="s">
+        <v>248</v>
+      </c>
+      <c r="B45" s="18" t="s">
+        <v>16</v>
+      </c>
+      <c r="C45" s="18"/>
+      <c r="D45" s="18" t="s">
+        <v>291</v>
+      </c>
+      <c r="E45" s="18" t="s">
+        <v>349</v>
+      </c>
+    </row>
+    <row r="46" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A46" s="18" t="s">
+        <v>60</v>
+      </c>
+      <c r="B46" s="18" t="s">
+        <v>281</v>
+      </c>
+      <c r="C46" s="18" t="s">
+        <v>298</v>
+      </c>
+      <c r="D46" s="18" t="s">
+        <v>299</v>
+      </c>
+      <c r="E46" s="18" t="s">
+        <v>300</v>
+      </c>
+    </row>
+    <row r="47" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A47" s="18" t="s">
+        <v>64</v>
+      </c>
+      <c r="B47" s="18" t="s">
+        <v>281</v>
+      </c>
+      <c r="C47" s="18" t="s">
+        <v>301</v>
+      </c>
+      <c r="D47" s="18" t="s">
+        <v>299</v>
+      </c>
+      <c r="E47" s="18" t="s">
+        <v>302</v>
+      </c>
+    </row>
+    <row r="48" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A48" s="18" t="s">
+        <v>67</v>
+      </c>
+      <c r="B48" s="18" t="s">
+        <v>281</v>
+      </c>
+      <c r="C48" s="18" t="s">
+        <v>303</v>
+      </c>
+      <c r="D48" s="18" t="s">
+        <v>299</v>
+      </c>
+      <c r="E48" s="18" t="s">
+        <v>304</v>
+      </c>
+      <c r="F48" s="18"/>
+      <c r="G48" s="18"/>
+    </row>
+    <row r="49" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A49" s="18" t="s">
+        <v>71</v>
+      </c>
+      <c r="B49" s="18" t="s">
+        <v>281</v>
+      </c>
+      <c r="C49" s="18" t="s">
+        <v>301</v>
+      </c>
+      <c r="D49" s="18" t="s">
+        <v>299</v>
+      </c>
+      <c r="E49" s="18" t="s">
+        <v>305</v>
+      </c>
+      <c r="F49" s="18"/>
+      <c r="G49" s="18"/>
+    </row>
+    <row r="50" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A50" s="18" t="s">
+        <v>75</v>
+      </c>
+      <c r="B50" s="18" t="s">
+        <v>281</v>
+      </c>
+      <c r="C50" s="18" t="s">
+        <v>301</v>
+      </c>
+      <c r="D50" s="18" t="s">
+        <v>299</v>
+      </c>
+      <c r="E50" s="18" t="s">
+        <v>355</v>
+      </c>
+      <c r="F50" s="18"/>
+      <c r="G50" s="18"/>
+    </row>
+    <row r="51" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A51" s="18" t="s">
+        <v>76</v>
+      </c>
+      <c r="B51" s="18" t="s">
+        <v>281</v>
+      </c>
+      <c r="C51" s="18" t="s">
+        <v>9</v>
+      </c>
+      <c r="D51" s="18" t="s">
+        <v>299</v>
+      </c>
+      <c r="E51" s="18" t="s">
+        <v>356</v>
+      </c>
+      <c r="F51" s="18"/>
+      <c r="G51" s="18"/>
+    </row>
+    <row r="52" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A52" s="18" t="s">
+        <v>77</v>
+      </c>
+      <c r="B52" s="18" t="s">
+        <v>281</v>
+      </c>
+      <c r="C52" s="18" t="s">
+        <v>351</v>
+      </c>
+      <c r="D52" s="18" t="s">
+        <v>299</v>
+      </c>
+      <c r="E52" s="18" t="s">
+        <v>353</v>
+      </c>
+      <c r="F52" s="18"/>
+      <c r="G52" s="18"/>
+    </row>
+    <row r="53" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A53" s="18" t="s">
+        <v>78</v>
+      </c>
+      <c r="B53" s="18" t="s">
+        <v>281</v>
+      </c>
+      <c r="C53" s="18" t="s">
+        <v>351</v>
+      </c>
+      <c r="D53" s="18" t="s">
+        <v>299</v>
+      </c>
+      <c r="E53" s="18" t="s">
+        <v>352</v>
+      </c>
+      <c r="F53" s="18"/>
+      <c r="G53" s="18"/>
+    </row>
+    <row r="54" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A54" s="18" t="s">
+        <v>74</v>
+      </c>
+      <c r="B54" s="18" t="s">
+        <v>267</v>
+      </c>
+      <c r="C54" s="18" t="s">
+        <v>9</v>
+      </c>
+      <c r="D54" s="18" t="s">
+        <v>270</v>
+      </c>
+      <c r="E54" s="18" t="s">
+        <v>271</v>
+      </c>
+      <c r="F54" s="18"/>
+      <c r="G54" s="18"/>
+    </row>
+    <row r="55" spans="1:7" ht="43.2" x14ac:dyDescent="0.3">
+      <c r="A55" s="18" t="s">
+        <v>22</v>
+      </c>
+      <c r="B55" s="18" t="s">
+        <v>16</v>
+      </c>
+      <c r="C55" s="18" t="s">
+        <v>276</v>
+      </c>
+      <c r="D55" s="18" t="s">
+        <v>270</v>
+      </c>
+      <c r="E55" s="18" t="s">
+        <v>277</v>
+      </c>
+      <c r="F55" s="18"/>
+      <c r="G55" s="18"/>
+    </row>
+    <row r="56" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A56" s="18" t="s">
+        <v>17</v>
+      </c>
+      <c r="B56" s="18" t="s">
+        <v>272</v>
+      </c>
+      <c r="C56" s="18" t="s">
+        <v>273</v>
+      </c>
+      <c r="D56" s="18" t="s">
+        <v>270</v>
+      </c>
+      <c r="E56" s="18" t="s">
+        <v>278</v>
+      </c>
+      <c r="F56" s="18"/>
+      <c r="G56" s="18"/>
+    </row>
+    <row r="57" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A57" s="18" t="s">
+        <v>31</v>
+      </c>
+      <c r="B57" s="18" t="s">
+        <v>16</v>
+      </c>
+      <c r="C57" s="18" t="s">
+        <v>9</v>
+      </c>
+      <c r="D57" s="18" t="s">
+        <v>270</v>
+      </c>
+      <c r="E57" s="18" t="s">
+        <v>279</v>
+      </c>
+      <c r="F57" s="18"/>
+      <c r="G57" s="18"/>
+    </row>
+    <row r="58" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A58" s="18" t="s">
+        <v>25</v>
+      </c>
+      <c r="B58" s="18" t="s">
+        <v>272</v>
+      </c>
+      <c r="C58" s="18" t="s">
+        <v>273</v>
+      </c>
+      <c r="D58" s="18" t="s">
+        <v>270</v>
+      </c>
+      <c r="E58" s="18" t="s">
+        <v>280</v>
+      </c>
+      <c r="F58" s="18"/>
+      <c r="G58" s="18"/>
+    </row>
+    <row r="59" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A59" s="18" t="s">
+        <v>30</v>
+      </c>
+      <c r="B59" s="18" t="s">
+        <v>16</v>
+      </c>
+      <c r="C59" s="18" t="s">
+        <v>290</v>
+      </c>
+      <c r="D59" s="18" t="s">
+        <v>270</v>
+      </c>
+      <c r="E59" s="18" t="s">
+        <v>358</v>
+      </c>
+      <c r="F59" s="18"/>
+      <c r="G59" s="18"/>
+    </row>
+    <row r="60" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A60" s="18" t="s">
+        <v>32</v>
+      </c>
+      <c r="B60" s="18" t="s">
+        <v>16</v>
+      </c>
+      <c r="C60" s="18"/>
+      <c r="D60" s="18" t="s">
+        <v>270</v>
+      </c>
+      <c r="E60" s="18"/>
+      <c r="F60" s="18"/>
+      <c r="G60" s="18"/>
+    </row>
+    <row r="61" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A61" s="18"/>
+      <c r="B61" s="18"/>
+      <c r="C61" s="18"/>
+      <c r="D61" s="18"/>
+      <c r="E61" s="18"/>
+      <c r="F61" s="18"/>
+      <c r="G61" s="18"/>
+    </row>
+    <row r="62" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A62" s="18"/>
+      <c r="B62" s="18"/>
+      <c r="C62" s="18"/>
+      <c r="D62" s="18"/>
+      <c r="E62" s="18"/>
+      <c r="F62" s="18"/>
+      <c r="G62" s="18"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>